<commit_message>
Move extraction to Opus 5.5 medium: effort sweep, nine re-extractions, one-version cockpit
- Runner defaults to Claude Opus 5.5 at medium effort; the 22 September sweep
  (Opus medium/high, GPT-6-Sol high/xhigh; three deals, blind graded) found no
  reliable gain from higher effort.
- extraction/ holds Opus 5.5 medium extractions of all nine deals under the
  unchanged v1.13.2 instruction; receipts in the re-extraction packet. The
  replaced workbooks are archived outside the checkout and recoverable here
  at 03d59b1.
- The cockpit shows one Opus 5.5 version per deal; findings keyed to old
  workbook rows were removed, the Datalink F9 ruling and Mac-Gray R01 kept.
- Austin's R01 decision recorded: bidder-commitment changes are same-price
  Bids; the target termination fee stays in a dated Note.
- Checker requires all seventeen v1.13.2 Deal facts fields; stale files, dead
  code and superseded build assets retired.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/extraction/kraton.xlsx
+++ b/extraction/kraton.xlsx
@@ -13,9 +13,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Deal facts" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Deal ledger'!$A$1:$V$75</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rounds'!$A$1:$J$5</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Questions'!$A$1:$G$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Deal ledger'!$A$1:$V$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Rounds'!$A$1:$J$4</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Questions'!$A$1:$G$9</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Deal facts'!$A$1:$B$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +25,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="MM/DD/YYYY"/>
   </numFmts>
   <fonts count="2">
@@ -439,21 +439,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V75"/>
+  <dimension ref="A1:V74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="22" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
     <col width="7" customWidth="1" min="7" max="7"/>
     <col width="9" customWidth="1" min="8" max="8"/>
     <col width="9" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
-    <col width="11" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
     <col width="7" customWidth="1" min="13" max="13"/>
     <col width="20" customWidth="1" min="14" max="14"/>
     <col width="8" customWidth="1" min="15" max="15"/>
@@ -461,9 +461,9 @@
     <col width="60" customWidth="1" min="17" max="17"/>
     <col width="10" customWidth="1" min="18" max="18"/>
     <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="11" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
+    <col width="11" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -589,7 +589,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>J.P. Morgan (target)</t>
+          <t>J.P. Morgan</t>
         </is>
       </c>
       <c r="D2" s="2" t="n"/>
@@ -614,7 +614,7 @@
       <c r="O2" s="2" t="n"/>
       <c r="P2" s="2" t="inlineStr">
         <is>
-          <t>Kraton's financial adviser; attended the Board's September, November and December 2020 strategy meetings and executed the corporate development plan. Board formally approved its engagement 08/11/2021; engagement letter dated 08/13/2021 (p. 6).</t>
+          <t>Kraton's financial adviser; attended the September, November and December 2020 strategy meetings. Board formally approved its engagement for the sale on 08/11/2021; engagement letter dated 08/13/2021 (p. 6); fee about $32 million, mostly contingent on completion (p. 52).</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
@@ -645,7 +645,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
+          <t>Kraton</t>
         </is>
       </c>
       <c r="D3" s="2" t="n"/>
@@ -670,7 +670,7 @@
       <c r="O3" s="2" t="n"/>
       <c r="P3" s="2" t="inlineStr">
         <is>
-          <t>Board authorizes a corporate development plan: acquire or combine with other parties' polymer businesses and/or sell the crude sulfate turpentine (CST) business, part of the chemical segment. Not a whole-company sale. Ref: $26.25 close 12/14/2020.</t>
+          <t>Board authorizes a corporate development plan: grow the polymer business by acquiring or combining with other parties' polymer businesses (Kraton as buyer; talks with Parties A and B, who declined) and/or sell the CST business, part of the chemical segment. Not a whole-company sale. Ref: $26.25 close 12/14/2020.</t>
         </is>
       </c>
       <c r="Q3" s="2" t="inlineStr">
@@ -678,11 +678,7 @@
           <t>“On December 14, 2020, the date on which the Board authorized Kraton to pursue the corporate development plan” (p. 32)</t>
         </is>
       </c>
-      <c r="R3" s="2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R3" s="2" t="n"/>
       <c r="S3" s="2" t="n"/>
       <c r="T3" s="3" t="n">
         <v>44179</v>
@@ -700,12 +696,12 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>late 2020 – early 2021</t>
+          <t>late 2020 and early 2021</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Party C</t>
+          <t>Parties C, D, E and G</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -730,13 +726,13 @@
       <c r="K4" s="2" t="n"/>
       <c r="L4" s="2" t="n"/>
       <c r="M4" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N4" s="2" t="n"/>
       <c r="O4" s="2" t="n"/>
       <c r="P4" s="2" t="inlineStr">
         <is>
-          <t>Target-initiated: Kraton management and J.P. Morgan discussed a sale of the CST business (segment only) under the corporate development plan. Party C said it might be interested, subject to further diligence and analysis. Window: after 12/14/2020 authorization, before 05/20/2021 Board review.</t>
+          <t>Target-initiated: management and J.P. Morgan discussed a sale of the CST business (segment only) with each; each said it might be interested, subject to further diligence and analysis. Window runs from the 12/14/2020 authorization to the 05/20/2021 Board review.</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
@@ -744,7 +740,11 @@
           <t>“Each of Party C, Party D, Party E, and Party G informed Kraton that they might be interested in acquiring Kraton’s CST business, subject to further diligence and analysis.” (p. 32)</t>
         </is>
       </c>
-      <c r="R4" s="2" t="n"/>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S4" s="2" t="n"/>
       <c r="T4" s="3" t="n">
         <v>44257</v>
@@ -762,12 +762,12 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>late 2020 – early 2021</t>
+          <t>late 2020 and early 2021</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Party D</t>
+          <t>Party F</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -798,15 +798,19 @@
       <c r="O5" s="2" t="n"/>
       <c r="P5" s="2" t="inlineStr">
         <is>
-          <t>Target-initiated: Kraton management and J.P. Morgan discussed a sale of the CST business (segment only) under the corporate development plan. Party D said it might be interested, subject to further diligence and analysis. Window: after 12/14/2020 authorization, before 05/20/2021 Board review.</t>
+          <t>Target-initiated discussion of a sale of the CST business; Party F said it was not interested. Never entered.</t>
         </is>
       </c>
       <c r="Q5" s="2" t="inlineStr">
         <is>
-          <t>“Each of Party C, Party D, Party E, and Party G informed Kraton that they might be interested in acquiring Kraton’s CST business, subject to further diligence and analysis.” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R5" s="2" t="n"/>
+          <t>“Party F informed Kraton that it was not interested in acquiring Kraton’s CST business.” (p. 32)</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S5" s="2" t="n"/>
       <c r="T5" s="3" t="n">
         <v>44257</v>
@@ -824,22 +828,18 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>late 2020 – early 2021</t>
+          <t>05/20/2021</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Party E</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>King &amp; Spalding LLP</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="n"/>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Adviser</t>
         </is>
       </c>
       <c r="F6" s="2" t="n">
@@ -853,28 +853,26 @@
       <c r="J6" s="2" t="n"/>
       <c r="K6" s="2" t="n"/>
       <c r="L6" s="2" t="n"/>
-      <c r="M6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M6" s="2" t="n"/>
       <c r="N6" s="2" t="n"/>
       <c r="O6" s="2" t="n"/>
       <c r="P6" s="2" t="inlineStr">
         <is>
-          <t>Target-initiated: Kraton management and J.P. Morgan discussed a sale of the CST business (segment only) under the corporate development plan. Party E said it might be interested, subject to further diligence and analysis. Window: after 12/14/2020 authorization, before 05/20/2021 Board review.</t>
+          <t>Kraton's legal adviser; first shown acting at the 05/20/2021 Board meeting; later reviewed fiduciary duties and drafted and negotiated the merger agreement.</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>“Each of Party C, Party D, Party E, and Party G informed Kraton that they might be interested in acquiring Kraton’s CST business, subject to further diligence and analysis.” (p. 32)</t>
+          <t>“Representatives of J.P. Morgan and King &amp; Spalding LLP, Kraton’s legal advisor, also participated in the meeting.” (p. 32)</t>
         </is>
       </c>
       <c r="R6" s="2" t="n"/>
       <c r="S6" s="2" t="n"/>
       <c r="T6" s="3" t="n">
-        <v>44257</v>
+        <v>44336</v>
       </c>
       <c r="U6" s="3" t="n">
-        <v>44179</v>
+        <v>44336</v>
       </c>
       <c r="V6" s="3" t="n">
         <v>44336</v>
@@ -886,22 +884,18 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>late 2020 – early 2021</t>
+          <t>05/20/2021</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Party G</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Kraton</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="n"/>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Target sale decision</t>
         </is>
       </c>
       <c r="F7" s="2" t="n">
@@ -915,28 +909,26 @@
       <c r="J7" s="2" t="n"/>
       <c r="K7" s="2" t="n"/>
       <c r="L7" s="2" t="n"/>
-      <c r="M7" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M7" s="2" t="n"/>
       <c r="N7" s="2" t="n"/>
       <c r="O7" s="2" t="n"/>
       <c r="P7" s="2" t="inlineStr">
         <is>
-          <t>Target-initiated: Kraton management and J.P. Morgan discussed a sale of the CST business (segment only) under the corporate development plan. Party G said it might be interested, subject to further diligence and analysis. Window: after 12/14/2020 authorization, before 05/20/2021 Board review.</t>
+          <t>Board decides to explore a potential sale of all of Kraton after the corporate development plan gained no momentum; directs management and J.P. Morgan to prepare a buyer list, timeline and process for review the following week. Ref: $33.82 close 05/20/2021.</t>
         </is>
       </c>
       <c r="Q7" s="2" t="inlineStr">
         <is>
-          <t>“Each of Party C, Party D, Party E, and Party G informed Kraton that they might be interested in acquiring Kraton’s CST business, subject to further diligence and analysis.” (p. 32)</t>
+          <t>“the Board determined that it would be in the best interests of Kraton and its stockholders to explore the potential sale of all of Kraton” (p. 33)</t>
         </is>
       </c>
       <c r="R7" s="2" t="n"/>
       <c r="S7" s="2" t="n"/>
       <c r="T7" s="3" t="n">
-        <v>44257</v>
+        <v>44336</v>
       </c>
       <c r="U7" s="3" t="n">
-        <v>44179</v>
+        <v>44336</v>
       </c>
       <c r="V7" s="3" t="n">
         <v>44336</v>
@@ -948,12 +940,12 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>late 2020 – early 2021</t>
+          <t>05/20/2021</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Party F</t>
+          <t>Parties C, D, E and G</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -963,7 +955,7 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Contact</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F8" s="2" t="n">
@@ -978,27 +970,31 @@
       <c r="K8" s="2" t="n"/>
       <c r="L8" s="2" t="n"/>
       <c r="M8" s="2" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="N8" s="2" t="n"/>
       <c r="O8" s="2" t="n"/>
       <c r="P8" s="2" t="inlineStr">
         <is>
-          <t>Target-initiated discussion of a sale of the CST business (segment only). Party F declined: not interested. Never entered. Window: after 12/14/2020 authorization, before 05/20/2021 Board review.</t>
+          <t>Admission decision: Board will review the CST proposals of C, D, E and G alongside any whole-company proposals, keeping them in the process as segment-only participants (treated as their entry). J.P. Morgan expected clarity on their interest by mid-June; management met each in June.</t>
         </is>
       </c>
       <c r="Q8" s="2" t="inlineStr">
         <is>
-          <t>“Party F informed Kraton that it was not interested in acquiring Kraton’s CST business.” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R8" s="2" t="n"/>
+          <t>“The Board also informed Kraton’s senior management and J.P. Morgan that it would review any proposals submitted by Party C, Party D, Party E, and Party G” (p. 33)</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S8" s="2" t="n"/>
       <c r="T8" s="3" t="n">
-        <v>44257</v>
+        <v>44336</v>
       </c>
       <c r="U8" s="3" t="n">
-        <v>44179</v>
+        <v>44336</v>
       </c>
       <c r="V8" s="3" t="n">
         <v>44336</v>
@@ -1010,25 +1006,25 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>05/20/2021</t>
+          <t>05/24/2021</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>King &amp; Spalding LLP (target)</t>
+          <t>Kraton</t>
         </is>
       </c>
       <c r="D9" s="2" t="n"/>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Adviser</t>
+          <t>Round opened</t>
         </is>
       </c>
       <c r="F9" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H9" s="2" t="n"/>
       <c r="I9" s="2" t="n"/>
@@ -1040,24 +1036,28 @@
       <c r="O9" s="2" t="n"/>
       <c r="P9" s="2" t="inlineStr">
         <is>
-          <t>Kraton's legal adviser; first shown acting at the 05/20/2021 Board meeting; advised on fiduciary duties and the merger agreement through signing.</t>
+          <t>Board reviews a buyer list (strategic, financial and sponsors with chemical/polymer portfolio companies, including Party A, Party B's parent and Parent), a two-phase process with initial indications on mainly public information in the third week of June, and directs outreach to 14. Ref: $34.33 close.</t>
         </is>
       </c>
       <c r="Q9" s="2" t="inlineStr">
         <is>
-          <t>“Representatives of J.P. Morgan and King &amp; Spalding LLP, Kraton’s legal advisor, also participated in the meeting.” (p. 32)</t>
-        </is>
-      </c>
-      <c r="R9" s="2" t="n"/>
+          <t>“the Board directed Kraton’s senior management to work with J.P. Morgan to contact the 14 possible acquirers that were discussed at the meeting” (p. 33)</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>Q2</t>
+        </is>
+      </c>
       <c r="S9" s="2" t="n"/>
       <c r="T9" s="3" t="n">
-        <v>44336</v>
+        <v>44340</v>
       </c>
       <c r="U9" s="3" t="n">
-        <v>44336</v>
+        <v>44340</v>
       </c>
       <c r="V9" s="3" t="n">
-        <v>44336</v>
+        <v>44340</v>
       </c>
     </row>
     <row r="10">
@@ -1066,42 +1066,60 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>05/20/2021</t>
+          <t>by 07/02/2021</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="n"/>
+          <t>Party C</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Target sale decision</t>
+          <t>Other-scope bid</t>
         </is>
       </c>
       <c r="F10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H10" s="2" t="n"/>
       <c r="I10" s="2" t="n"/>
-      <c r="J10" s="2" t="n"/>
-      <c r="K10" s="2" t="n"/>
-      <c r="L10" s="2" t="n"/>
-      <c r="M10" s="2" t="n"/>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N10" s="2" t="n"/>
       <c r="O10" s="2" t="n"/>
       <c r="P10" s="2" t="inlineStr">
         <is>
-          <t>Corporate development plan had gained no momentum; Board decides to explore a sale of all of Kraton, orders a buyer list and timeline for review the next week, and will weigh any CST proposals (Parties C, D, E, G) against whole-company proposals. Ref: $33.82 close 05/20/2021.</t>
+          <t>Unclear: no conditions reported. Proposes to buy a portion of the CST business for $100 million (total, not per share). First proposal after the 05/20 Board review, which reported only interest.</t>
         </is>
       </c>
       <c r="Q10" s="2" t="inlineStr">
         <is>
-          <t>“the Board determined that it would be in the best interests of Kraton and its stockholders to explore the potential sale of all of Kraton” (p. 33)</t>
+          <t>“Party C proposed acquiring a portion of Kraton’s CST business for $100 million” (p. 35)</t>
         </is>
       </c>
       <c r="R10" s="2" t="inlineStr">
@@ -1111,13 +1129,13 @@
       </c>
       <c r="S10" s="2" t="n"/>
       <c r="T10" s="3" t="n">
-        <v>44336</v>
+        <v>44357</v>
       </c>
       <c r="U10" s="3" t="n">
         <v>44336</v>
       </c>
       <c r="V10" s="3" t="n">
-        <v>44336</v>
+        <v>44379</v>
       </c>
     </row>
     <row r="11">
@@ -1126,18 +1144,22 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>05/24/2021</t>
+          <t>by 07/02/2021</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
-        </is>
-      </c>
-      <c r="D11" s="2" t="n"/>
+          <t>Party G</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Round opened</t>
+          <t>Other-scope bid</t>
         </is>
       </c>
       <c r="F11" s="2" t="n">
@@ -1148,20 +1170,34 @@
       </c>
       <c r="H11" s="2" t="n"/>
       <c r="I11" s="2" t="n"/>
-      <c r="J11" s="2" t="n"/>
-      <c r="K11" s="2" t="n"/>
-      <c r="L11" s="2" t="n"/>
-      <c r="M11" s="2" t="n"/>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N11" s="2" t="n"/>
       <c r="O11" s="2" t="n"/>
       <c r="P11" s="2" t="inlineStr">
         <is>
-          <t>Board reviews list of strategic, financial and sponsor-with-portfolio-company buyers (incl. Party A, Party B's parent, Parent); plans two-phase process: IOIs on public information in third week of June, highest-value bidders to a second round. Outreach began end of May. Ref: $34.33 close 05/24/2021.</t>
+          <t>Unclear: price subject to unspecified adjustments; no other condition reported. Proposes to buy a portion of the CST business for $330 million (total, not per share).</t>
         </is>
       </c>
       <c r="Q11" s="2" t="inlineStr">
         <is>
-          <t>“the Board directed Kraton’s senior management to work with J.P. Morgan to contact the 14 possible acquirers that were discussed at the meeting to explore their interest” (p. 33)</t>
+          <t>“Party G proposed acquiring a portion of Kraton’s CST business for $330 million, subject to adjustments” (p. 35)</t>
         </is>
       </c>
       <c r="R11" s="2" t="inlineStr">
@@ -1171,13 +1207,13 @@
       </c>
       <c r="S11" s="2" t="n"/>
       <c r="T11" s="3" t="n">
-        <v>44340</v>
+        <v>44357</v>
       </c>
       <c r="U11" s="3" t="n">
-        <v>44340</v>
+        <v>44336</v>
       </c>
       <c r="V11" s="3" t="n">
-        <v>44340</v>
+        <v>44379</v>
       </c>
     </row>
     <row r="12">
@@ -1191,12 +1227,12 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>14 listed possible acquirers</t>
+          <t>Party A</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Unknown</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
@@ -1216,13 +1252,13 @@
       <c r="K12" s="2" t="n"/>
       <c r="L12" s="2" t="n"/>
       <c r="M12" s="2" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="N12" s="2" t="n"/>
       <c r="O12" s="2" t="n"/>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>Target-initiated outreach by management/J.P. Morgan; includes Party A, Party B's parent and Parent. Told whole-company bids preferred but stock deals or segment sales would be considered. Five contacted parties declined NDAs; exact arithmetic: 14 − 5 = 9 signed.</t>
+          <t>Target-initiated outreach; Party A was on the 14-party list (p. 33). Earlier (late 2020–early 2021) Party A had declined Kraton's approach to buy its polymer business (p. 32). Parties were told a whole-company bid was preferred but any value-maximizing proposal, including stock or segment deals, would be considered.</t>
         </is>
       </c>
       <c r="Q12" s="2" t="inlineStr">
@@ -1230,11 +1266,7 @@
           <t>“contacted each of the 14 parties discussed with the Board at its May 24, 2021 meeting to explore the parties’ respective interest in a potential acquisition of Kraton” (p. 34)</t>
         </is>
       </c>
-      <c r="R12" s="2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+      <c r="R12" s="2" t="n"/>
       <c r="S12" s="2" t="n"/>
       <c r="T12" s="3" t="n">
         <v>44358</v>
@@ -1257,7 +1289,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Unnamed strategic inbound party</t>
+          <t>Parent (DL Chemical Co., Ltd.)</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1267,7 +1299,7 @@
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Bidder interest</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="F13" s="2" t="n">
@@ -1288,12 +1320,12 @@
       <c r="O13" s="2" t="n"/>
       <c r="P13" s="2" t="inlineStr">
         <is>
-          <t>Inbound inquiry to J.P. Morgan by a strategic party not on the Board's list; it later signed an NDA (counted in the six strategic signers, next row).</t>
+          <t>Target-initiated outreach; Parent was on the 14-party list (p. 33). Parent, a Korean petrochemical company owned by DL Holdings, bought Kraton's Cariflex business for $530 million in March 2020 (p. 29).</t>
         </is>
       </c>
       <c r="Q13" s="2" t="inlineStr">
         <is>
-          <t>“a potential strategic acquirer that was not included on the list of possible acquirers made an “inbound” inquiry and contacted representatives of J.P. Morgan regarding a potential acquisition of Kraton” (p. 34)</t>
+          <t>“contacted each of the 14 parties discussed with the Board at its May 24, 2021 meeting to explore the parties’ respective interest in a potential acquisition of Kraton” (p. 34)</t>
         </is>
       </c>
       <c r="R13" s="2" t="n"/>
@@ -1314,22 +1346,22 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>by late June 2021</t>
+          <t>end of May and June 2021</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>6 strategic NDA signers</t>
+          <t>Party B's parent company</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>NDA signed</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="F14" s="2" t="n">
@@ -1344,23 +1376,23 @@
       <c r="K14" s="2" t="n"/>
       <c r="L14" s="2" t="n"/>
       <c r="M14" s="2" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="N14" s="2" t="n"/>
       <c r="O14" s="2" t="n"/>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>Stated total 10 NDAs: 6 strategic (incl. inbound party), 4 financial; standstills lapse on an announced definitive agreement. June preliminary management meetings (near-term performance, innovation projects) for 9 signers (5 strategic, 4 financial). Party A, Parent, Party J, Party K presumed members, not stated.</t>
+          <t>Target-initiated outreach; on the 14-party list (p. 33). Party B (strategic) had declined a polymer combination earlier. Whether its parent signed a confidentiality agreement or was among the five decliners is not reported.</t>
         </is>
       </c>
       <c r="Q14" s="2" t="inlineStr">
         <is>
-          <t>“By late June 2021, Kraton had entered into confidentiality agreements with 10 parties (including the party that made the “inbound” inquiry), six of which parties were potential strategic acquirers” (p. 34)</t>
+          <t>“contacted each of the 14 parties discussed with the Board at its May 24, 2021 meeting to explore the parties’ respective interest in a potential acquisition of Kraton” (p. 34)</t>
         </is>
       </c>
       <c r="R14" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="S14" s="2" t="n"/>
@@ -1380,22 +1412,22 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>by late June 2021</t>
+          <t>end of May and June 2021</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>4 financial NDA signers</t>
+          <t>11 other listed parties</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Unknown</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>NDA signed</t>
+          <t>Contact</t>
         </is>
       </c>
       <c r="F15" s="2" t="n">
@@ -1410,23 +1442,23 @@
       <c r="K15" s="2" t="n"/>
       <c r="L15" s="2" t="n"/>
       <c r="M15" s="2" t="n">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="N15" s="2" t="n"/>
       <c r="O15" s="2" t="n"/>
       <c r="P15" s="2" t="inlineStr">
         <is>
-          <t>Part of the stated 10 NDAs (6 strategic, 4 financial), standstills included; all four attended June preliminary management meetings. Party H and Party I presumed members, not stated.</t>
+          <t>Count: 11 = 14 listed − Party A, Parent, Party B's parent. Mix of strategic and financial, split not given. With the inbound party, 15 contacted = 10 confidentiality signers + 5 decliners (p. 34); Parties H, I and probably J, K are among these 11.</t>
         </is>
       </c>
       <c r="Q15" s="2" t="inlineStr">
         <is>
-          <t>“six of which parties were potential strategic acquirers and four of which were potential financial acquirers” (p. 34)</t>
+          <t>“contacted each of the 14 parties discussed with the Board at its May 24, 2021 meeting to explore the parties’ respective interest in a potential acquisition of Kraton” (p. 34)</t>
         </is>
       </c>
       <c r="R15" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="S15" s="2" t="n"/>
@@ -1446,12 +1478,12 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>June 2021</t>
+          <t>end of May and June 2021</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Parties C, D, E and G</t>
+          <t>Unnamed inbound strategic party</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1461,7 +1493,7 @@
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Bidder interest</t>
         </is>
       </c>
       <c r="F16" s="2" t="n">
@@ -1476,18 +1508,18 @@
       <c r="K16" s="2" t="n"/>
       <c r="L16" s="2" t="n"/>
       <c r="M16" s="2" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="N16" s="2" t="n"/>
       <c r="O16" s="2" t="n"/>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>Kraton admits the four CST-interested parties to preliminary management meetings on a CST-only sale; treated as their entry (segment scope, not whole company). Window ends 06/17/2021 because Party E withdrew 06/18/2021.</t>
+          <t>Inbound inquiry to J.P. Morgan about acquiring Kraton, no price; not on the 14-party list. Signed a confidentiality agreement by late June (inside the strategic cohort); it is not Party A or Parent (both on the list) and may be Party J, Party K or an unnamed signer.</t>
         </is>
       </c>
       <c r="Q16" s="2" t="inlineStr">
         <is>
-          <t>“Kraton’s senior management also participated in preliminary management meetings with Party C, Party D, Party E, and Party G regarding the potential sale of Kraton’s CST business.” (p. 34)</t>
+          <t>“a potential strategic acquirer that was not included on the list of possible acquirers made an “inbound” inquiry and contacted representatives of J.P. Morgan” (p. 34)</t>
         </is>
       </c>
       <c r="R16" s="2" t="inlineStr">
@@ -1500,10 +1532,10 @@
         <v>44358</v>
       </c>
       <c r="U16" s="3" t="n">
-        <v>44348</v>
+        <v>44336</v>
       </c>
       <c r="V16" s="3" t="n">
-        <v>44364</v>
+        <v>44377</v>
       </c>
     </row>
     <row r="17">
@@ -1512,18 +1544,22 @@
       </c>
       <c r="B17" s="2" t="inlineStr">
         <is>
-          <t>June 2021</t>
+          <t>by late June 2021</t>
         </is>
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="n"/>
+          <t>6 strategic confidentiality signers</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>Deadline set</t>
+          <t>NDA signed</t>
         </is>
       </c>
       <c r="F17" s="2" t="n">
@@ -1537,29 +1573,35 @@
       <c r="J17" s="2" t="n"/>
       <c r="K17" s="2" t="n"/>
       <c r="L17" s="2" t="n"/>
-      <c r="M17" s="2" t="n"/>
+      <c r="M17" s="2" t="n">
+        <v>6</v>
+      </c>
       <c r="N17" s="2" t="n"/>
       <c r="O17" s="2" t="n"/>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t>J.P. Morgan's process letter to every NDA signer asks for initial indications of interest by 06/29/2021; bars discussion of management's post-closing roles. Sent before the due date.</t>
+          <t>Count: 6 of 10 signers (p. 34), including the inbound party; by the contact accounting (15 contacted = 10 signers + 5 decliners) Party A, Parent, Party J and Party K are members. Standstills lapse on announcement of a definitive agreement. June preliminary management meetings with 5 strategic signers.</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
         <is>
-          <t>“circulated a process letter to each party that executed a confidentiality agreement that requested initial indications of interest be submitted by June 29, 2021” (p. 34)</t>
-        </is>
-      </c>
-      <c r="R17" s="2" t="n"/>
+          <t>“Kraton had entered into confidentiality agreements with 10 parties (including the party that made the “inbound” inquiry), six of which parties were potential strategic acquirers” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
       <c r="S17" s="2" t="n"/>
       <c r="T17" s="3" t="n">
-        <v>44361</v>
+        <v>44358</v>
       </c>
       <c r="U17" s="3" t="n">
-        <v>44348</v>
+        <v>44336</v>
       </c>
       <c r="V17" s="3" t="n">
-        <v>44375</v>
+        <v>44377</v>
       </c>
     </row>
     <row r="18">
@@ -1568,22 +1610,22 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>June 2021</t>
+          <t>by late June 2021</t>
         </is>
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>Unnamed strategic NDA signer</t>
+          <t>4 financial confidentiality signers</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Withdrew</t>
+          <t>NDA signed</t>
         </is>
       </c>
       <c r="F18" s="2" t="n">
@@ -1598,31 +1640,31 @@
       <c r="K18" s="2" t="n"/>
       <c r="L18" s="2" t="n"/>
       <c r="M18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N18" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
+        <v>4</v>
+      </c>
+      <c r="N18" s="2" t="n"/>
       <c r="O18" s="2" t="n"/>
       <c r="P18" s="2" t="inlineStr">
         <is>
-          <t>Declined the preliminary management meeting and said it was no longer interested. Type by exact arithmetic: 6 strategic signers − 5 strategic attendees = 1; all 4 financial attended.</t>
+          <t>Count: 4 of 10 signers (p. 34); Party H and Party I are members by the contact accounting. All four held June preliminary management meetings reviewing near-term performance and innovation projects, as did five strategic signers.</t>
         </is>
       </c>
       <c r="Q18" s="2" t="inlineStr">
         <is>
-          <t>“declined to participate in, this preliminary management meeting and informed representatives of J.P. Morgan that it was no longer interested in pursuing a potential transaction” (p. 34)</t>
-        </is>
-      </c>
-      <c r="R18" s="2" t="n"/>
+          <t>“six of which parties were potential strategic acquirers and four of which were potential financial acquirers” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Q3</t>
+        </is>
+      </c>
       <c r="S18" s="2" t="n"/>
       <c r="T18" s="3" t="n">
-        <v>44362</v>
+        <v>44358</v>
       </c>
       <c r="U18" s="3" t="n">
-        <v>44348</v>
+        <v>44340</v>
       </c>
       <c r="V18" s="3" t="n">
         <v>44377</v>
@@ -1634,22 +1676,18 @@
       </c>
       <c r="B19" s="2" t="inlineStr">
         <is>
-          <t>06/18/2021</t>
+          <t>June 2021</t>
         </is>
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>Party E</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Kraton</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="n"/>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Withdrew</t>
+          <t>Deadline set</t>
         </is>
       </c>
       <c r="F19" s="2" t="n">
@@ -1663,39 +1701,33 @@
       <c r="J19" s="2" t="n"/>
       <c r="K19" s="2" t="n"/>
       <c r="L19" s="2" t="n"/>
-      <c r="M19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N19" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
+      <c r="M19" s="2" t="n"/>
+      <c r="N19" s="2" t="n"/>
       <c r="O19" s="2" t="n"/>
       <c r="P19" s="2" t="inlineStr">
         <is>
-          <t>CST-only participant: no longer interested in acquiring the CST business. Never bid.</t>
+          <t>J.P. Morgan's process letter to every confidentiality signer asks for initial indications of interest by 06/29/2021 and bars discussions with management about post-closing roles (none occurred before signing).</t>
         </is>
       </c>
       <c r="Q19" s="2" t="inlineStr">
         <is>
-          <t>“On June 18, 2021, Party E informed Kraton that it was no longer interested in acquiring Kraton’s CST business.” (p. 34)</t>
+          <t>“circulated a process letter to each party that executed a confidentiality agreement that requested initial indications of interest be submitted by June 29, 2021” (p. 34)</t>
         </is>
       </c>
       <c r="R19" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S19" s="2" t="n"/>
       <c r="T19" s="3" t="n">
-        <v>44365</v>
+        <v>44361</v>
       </c>
       <c r="U19" s="3" t="n">
-        <v>44365</v>
+        <v>44348</v>
       </c>
       <c r="V19" s="3" t="n">
-        <v>44365</v>
+        <v>44375</v>
       </c>
     </row>
     <row r="20">
@@ -1704,12 +1736,12 @@
       </c>
       <c r="B20" s="2" t="inlineStr">
         <is>
-          <t>06/23/2021</t>
+          <t>June 2021</t>
         </is>
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>Party D</t>
+          <t>Unnamed strategic signer (declined meeting)</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1744,28 +1776,24 @@
       <c r="O20" s="2" t="n"/>
       <c r="P20" s="2" t="inlineStr">
         <is>
-          <t>CST-only participant: no longer interested in acquiring the CST business. Never bid.</t>
+          <t>Declined its preliminary management meeting and said it was no longer interested. Strategic by arithmetic: 6 strategic signers, 5 strategic met management.</t>
         </is>
       </c>
       <c r="Q20" s="2" t="inlineStr">
         <is>
-          <t>“On June 23, 2021, Party D informed Kraton that it was no longer interested in acquiring Kraton’s CST business.” (p. 34)</t>
-        </is>
-      </c>
-      <c r="R20" s="2" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
+          <t>“One party that executed a confidentiality agreement with Kraton was invited to, but declined to participate in, this preliminary management meeting” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="n"/>
       <c r="S20" s="2" t="n"/>
       <c r="T20" s="3" t="n">
-        <v>44370</v>
+        <v>44362</v>
       </c>
       <c r="U20" s="3" t="n">
-        <v>44370</v>
+        <v>44348</v>
       </c>
       <c r="V20" s="3" t="n">
-        <v>44370</v>
+        <v>44377</v>
       </c>
     </row>
     <row r="21">
@@ -1774,18 +1802,22 @@
       </c>
       <c r="B21" s="2" t="inlineStr">
         <is>
-          <t>06/29/2021</t>
+          <t>06/18/2021</t>
         </is>
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
-        </is>
-      </c>
-      <c r="D21" s="2" t="n"/>
+          <t>Party E</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Deadline</t>
+          <t>Withdrew</t>
         </is>
       </c>
       <c r="F21" s="2" t="n">
@@ -1799,33 +1831,39 @@
       <c r="J21" s="2" t="n"/>
       <c r="K21" s="2" t="n"/>
       <c r="L21" s="2" t="n"/>
-      <c r="M21" s="2" t="n"/>
-      <c r="N21" s="2" t="n"/>
+      <c r="M21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
       <c r="O21" s="2" t="n"/>
       <c r="P21" s="2" t="inlineStr">
         <is>
-          <t>Due date for first-round indications of interest. Four whole-company IOIs received by 07/02/2021; exact arrival days not stated.</t>
+          <t>Segment-only participant: no longer interested in acquiring the CST business. Never bid.</t>
         </is>
       </c>
       <c r="Q21" s="2" t="inlineStr">
         <is>
-          <t>“requested initial indications of interest be submitted by June 29, 2021” (p. 34)</t>
+          <t>“On June 18, 2021, Party E informed Kraton that it was no longer interested in acquiring Kraton’s CST business.” (p. 34)</t>
         </is>
       </c>
       <c r="R21" s="2" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="S21" s="2" t="n"/>
       <c r="T21" s="3" t="n">
-        <v>44376</v>
+        <v>44365</v>
       </c>
       <c r="U21" s="3" t="n">
-        <v>44376</v>
+        <v>44365</v>
       </c>
       <c r="V21" s="3" t="n">
-        <v>44376</v>
+        <v>44365</v>
       </c>
     </row>
     <row r="22">
@@ -1834,12 +1872,12 @@
       </c>
       <c r="B22" s="2" t="inlineStr">
         <is>
-          <t>by 07/02/2021</t>
+          <t>06/23/2021</t>
         </is>
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>Party A</t>
+          <t>Party D</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1849,7 +1887,7 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Withdrew</t>
         </is>
       </c>
       <c r="F22" s="2" t="n">
@@ -1858,52 +1896,44 @@
       <c r="G22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H22" s="4" t="n">
-        <v>42</v>
-      </c>
-      <c r="I22" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="J22" s="2" t="inlineStr">
+      <c r="H22" s="2" t="n"/>
+      <c r="I22" s="2" t="n"/>
+      <c r="J22" s="2" t="n"/>
+      <c r="K22" s="2" t="n"/>
+      <c r="L22" s="2" t="n"/>
+      <c r="M22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N22" s="2" t="n"/>
       <c r="O22" s="2" t="n"/>
       <c r="P22" s="2" t="inlineStr">
         <is>
-          <t>No conditions stated; IOI based primarily on public information, diligence still open. Non-binding first-round indication of interest, $42.00–$45.00 per share. Ref: $31.65 close 07/02/2021.</t>
+          <t>Segment-only participant: no longer interested in acquiring the CST business. Never bid.</t>
         </is>
       </c>
       <c r="Q22" s="2" t="inlineStr">
         <is>
-          <t>“Party A proposed $42.00 to $45.00, Party H, a financial acquirer, proposed $41.00 to $43.00, Parent proposed $41.00, and Party I, a financial acquirer, proposed $40.00.” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R22" s="2" t="n"/>
+          <t>“On June 23, 2021, Party D informed Kraton that it was no longer interested in acquiring Kraton’s CST business.” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S22" s="2" t="n"/>
       <c r="T22" s="3" t="n">
-        <v>44376</v>
+        <v>44370</v>
       </c>
       <c r="U22" s="3" t="n">
-        <v>44348</v>
+        <v>44370</v>
       </c>
       <c r="V22" s="3" t="n">
-        <v>44379</v>
+        <v>44370</v>
       </c>
     </row>
     <row r="23">
@@ -1912,22 +1942,18 @@
       </c>
       <c r="B23" s="2" t="inlineStr">
         <is>
-          <t>by 07/02/2021</t>
+          <t>06/29/2021</t>
         </is>
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>Party H</t>
-        </is>
-      </c>
-      <c r="D23" s="2" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
+          <t>Kraton</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="n"/>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Deadline</t>
         </is>
       </c>
       <c r="F23" s="2" t="n">
@@ -1936,52 +1962,38 @@
       <c r="G23" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H23" s="4" t="n">
-        <v>41</v>
-      </c>
-      <c r="I23" s="4" t="n">
-        <v>43</v>
-      </c>
-      <c r="J23" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="K23" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L23" s="2" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="M23" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="H23" s="2" t="n"/>
+      <c r="I23" s="2" t="n"/>
+      <c r="J23" s="2" t="n"/>
+      <c r="K23" s="2" t="n"/>
+      <c r="L23" s="2" t="n"/>
+      <c r="M23" s="2" t="n"/>
       <c r="N23" s="2" t="n"/>
       <c r="O23" s="2" t="n"/>
       <c r="P23" s="2" t="inlineStr">
         <is>
-          <t>No conditions stated; IOI based primarily on public information, diligence still open. First-round indication of interest, $41.00–$43.00 per share.</t>
+          <t>Due date for initial indications. Four whole-company indications were in hand by 07/02 (arrival days not given); Party J asked for more time. Board then set a further due date of 07/19 (#31).</t>
         </is>
       </c>
       <c r="Q23" s="2" t="inlineStr">
         <is>
-          <t>“Party A proposed $42.00 to $45.00, Party H, a financial acquirer, proposed $41.00 to $43.00, Parent proposed $41.00, and Party I, a financial acquirer, proposed $40.00.” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R23" s="2" t="n"/>
+          <t>“requested initial indications of interest be submitted by June 29, 2021” (p. 34)</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>Q4</t>
+        </is>
+      </c>
       <c r="S23" s="2" t="n"/>
       <c r="T23" s="3" t="n">
         <v>44376</v>
       </c>
       <c r="U23" s="3" t="n">
-        <v>44348</v>
+        <v>44376</v>
       </c>
       <c r="V23" s="3" t="n">
-        <v>44379</v>
+        <v>44376</v>
       </c>
     </row>
     <row r="24">
@@ -1995,7 +2007,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>Parent (DL Chemical)</t>
+          <t>Party A</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -2015,10 +2027,10 @@
         <v>1</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I24" s="4" t="n">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
@@ -2042,12 +2054,12 @@
       <c r="O24" s="2" t="n"/>
       <c r="P24" s="2" t="inlineStr">
         <is>
-          <t>No conditions stated; IOI based primarily on public information, diligence still open. First-round indication of interest at $41.00 per share. Parent (Korean petrochemical company, DL Holdings subsidiary) bought Kraton's Cariflex business in 2020 (p. 29).</t>
+          <t>Unclear: no stated conditions; first-round indication on mainly public information with diligence continuing. Initial indication of interest, whole company. Ref: $31.65 close 07/02/2021.</t>
         </is>
       </c>
       <c r="Q24" s="2" t="inlineStr">
         <is>
-          <t>“Party A proposed $42.00 to $45.00, Party H, a financial acquirer, proposed $41.00 to $43.00, Parent proposed $41.00, and Party I, a financial acquirer, proposed $40.00.” (p. 35)</t>
+          <t>“The per share purchase prices proposed by these parties were as follows: Party A proposed $42.00 to $45.00” (p. 35)</t>
         </is>
       </c>
       <c r="R24" s="2" t="n"/>
@@ -2073,7 +2085,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>Party I</t>
+          <t>Party H</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -2093,10 +2105,10 @@
         <v>1</v>
       </c>
       <c r="H25" s="4" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="I25" s="4" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
@@ -2120,12 +2132,12 @@
       <c r="O25" s="2" t="n"/>
       <c r="P25" s="2" t="inlineStr">
         <is>
-          <t>No conditions stated; IOI based primarily on public information, diligence still open. First-round indication of interest at $40.00 per share.</t>
+          <t>Unclear: no stated conditions; first-round indication on mainly public information with diligence continuing. Initial indication of interest, whole company.</t>
         </is>
       </c>
       <c r="Q25" s="2" t="inlineStr">
         <is>
-          <t>“Party A proposed $42.00 to $45.00, Party H, a financial acquirer, proposed $41.00 to $43.00, Parent proposed $41.00, and Party I, a financial acquirer, proposed $40.00.” (p. 35)</t>
+          <t>“Party H, a financial acquirer, proposed $41.00 to $43.00” (p. 35)</t>
         </is>
       </c>
       <c r="R25" s="2" t="n"/>
@@ -2151,7 +2163,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Party J</t>
+          <t>Parent (DL Chemical Co., Ltd.)</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2161,7 +2173,7 @@
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Did not submit</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F26" s="2" t="n">
@@ -2170,42 +2182,52 @@
       <c r="G26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H26" s="2" t="n"/>
-      <c r="I26" s="2" t="n"/>
-      <c r="J26" s="2" t="n"/>
-      <c r="K26" s="2" t="n"/>
-      <c r="L26" s="2" t="n"/>
+      <c r="H26" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="I26" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="J26" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
       <c r="M26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N26" s="2" t="inlineStr">
-        <is>
-          <t>Other stated reason</t>
-        </is>
-      </c>
+      <c r="N26" s="2" t="n"/>
       <c r="O26" s="2" t="n"/>
       <c r="P26" s="2" t="inlineStr">
         <is>
-          <t>No IOI by the 06/29/2021 due date; J told J.P. Morgan it intended to bid in mid-July. Treated as a presumed NDA signer eligible for round 1. Re-enters at #43.</t>
+          <t>Unclear: no stated conditions; first-round indication on mainly public information with diligence continuing. Initial indication of interest, whole company.</t>
         </is>
       </c>
       <c r="Q26" s="2" t="inlineStr">
         <is>
-          <t>“Party J, a strategic acquirer, informed representatives of J.P. Morgan that it intended to submit a proposal to acquire Kraton during the middle of July.” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R26" s="2" t="inlineStr">
-        <is>
-          <t>Q2; Q5</t>
-        </is>
-      </c>
+          <t>“Parent proposed $41.00, and Party I , a financial acquirer, proposed $40.00” (p. 35)</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="n"/>
       <c r="S26" s="2" t="n"/>
       <c r="T26" s="3" t="n">
         <v>44376</v>
       </c>
-      <c r="U26" s="2" t="n"/>
+      <c r="U26" s="3" t="n">
+        <v>44348</v>
+      </c>
       <c r="V26" s="3" t="n">
-        <v>44376</v>
+        <v>44379</v>
       </c>
     </row>
     <row r="27">
@@ -2219,17 +2241,17 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Party K</t>
+          <t>Party I</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Other-scope bid</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F27" s="2" t="n">
@@ -2238,8 +2260,12 @@
       <c r="G27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H27" s="2" t="n"/>
-      <c r="I27" s="2" t="n"/>
+      <c r="H27" s="4" t="n">
+        <v>40</v>
+      </c>
+      <c r="I27" s="4" t="n">
+        <v>40</v>
+      </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
@@ -2252,7 +2278,7 @@
       </c>
       <c r="L27" s="2" t="inlineStr">
         <is>
-          <t>Heavy</t>
+          <t>Unclear</t>
         </is>
       </c>
       <c r="M27" s="2" t="n">
@@ -2262,24 +2288,22 @@
       <c r="O27" s="2" t="n"/>
       <c r="P27" s="2" t="inlineStr">
         <is>
-          <t>Heavy: J.P. Morgan later reported this proposal subject to significant diligence and firm financing commitments (p. 37); only a standalone deal, no back-to-back polymer sale. Chemical segment at 9.0x–10.0x trailing-12-month (June 2021) segment adjusted EBITDA; no price stated.</t>
+          <t>Unclear: no stated conditions; first-round indication on mainly public information with diligence continuing. Initial indication of interest, whole company.</t>
         </is>
       </c>
       <c r="Q27" s="2" t="inlineStr">
         <is>
-          <t>“Party K, a potential strategic acquirer, proposed acquiring Kraton’s chemical segment.” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R27" s="2" t="inlineStr">
-        <is>
-          <t>Q2; Q3</t>
-        </is>
-      </c>
+          <t>“Parent proposed $41.00, and Party I , a financial acquirer, proposed $40.00” (p. 35)</t>
+        </is>
+      </c>
+      <c r="R27" s="2" t="n"/>
       <c r="S27" s="2" t="n"/>
       <c r="T27" s="3" t="n">
         <v>44376</v>
       </c>
-      <c r="U27" s="2" t="n"/>
+      <c r="U27" s="3" t="n">
+        <v>44348</v>
+      </c>
       <c r="V27" s="3" t="n">
         <v>44379</v>
       </c>
@@ -2290,12 +2314,12 @@
       </c>
       <c r="B28" s="2" t="inlineStr">
         <is>
-          <t>by 06/29/2021</t>
+          <t>by 07/02/2021</t>
         </is>
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Remaining strategic NDA signers (unnamed)</t>
+          <t>Party K</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2305,7 +2329,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Did not submit</t>
+          <t>Other-scope bid</t>
         </is>
       </c>
       <c r="F28" s="2" t="n">
@@ -2316,42 +2340,50 @@
       </c>
       <c r="H28" s="2" t="n"/>
       <c r="I28" s="2" t="n"/>
-      <c r="J28" s="2" t="n"/>
-      <c r="K28" s="2" t="n"/>
-      <c r="L28" s="2" t="n"/>
-      <c r="M28" s="2" t="n"/>
-      <c r="N28" s="2" t="inlineStr">
+      <c r="J28" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="O28" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="K28" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L28" s="2" t="inlineStr">
+        <is>
+          <t>Heavy</t>
+        </is>
+      </c>
+      <c r="M28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N28" s="2" t="n"/>
+      <c r="O28" s="2" t="n"/>
       <c r="P28" s="2" t="inlineStr">
         <is>
-          <t>Count: 1–5. Six strategic signers − 1 withdrawal (#17) = 5, less Party A, Parent, Party J (own row) and Party K if they were signers (likely, not stated): exactly 1 if all four were. No submission reported.</t>
+          <t>Heavy: J.P. Morgan said on 08/30 this proposal was still subject to significant diligence and firm financing commitments (p. 37). Chemical segment only, at 9.0x–10.0x segment adjusted EBITDA for the 12 months to June 2021; no dollar price; only if independent of any polymer sale.</t>
         </is>
       </c>
       <c r="Q28" s="2" t="inlineStr">
         <is>
-          <t>“By July 2, 2021, Kraton received four indications of interest as part of the first-round process that contemplated a potential acquisition of all of Kraton.” (p. 35)</t>
+          <t>“Party K, a potential strategic acquirer, proposed acquiring Kraton’s chemical segment. Party K did not propose a specific purchase price” (p. 35)</t>
         </is>
       </c>
       <c r="R28" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="S28" s="2" t="n"/>
       <c r="T28" s="3" t="n">
         <v>44376</v>
       </c>
-      <c r="U28" s="2" t="n"/>
+      <c r="U28" s="3" t="n">
+        <v>44348</v>
+      </c>
       <c r="V28" s="3" t="n">
-        <v>44376</v>
+        <v>44379</v>
       </c>
     </row>
     <row r="29">
@@ -2365,12 +2397,12 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Remaining financial NDA signers (unnamed)</t>
+          <t>1 unnamed strategic signer</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
@@ -2389,7 +2421,9 @@
       <c r="J29" s="2" t="n"/>
       <c r="K29" s="2" t="n"/>
       <c r="L29" s="2" t="n"/>
-      <c r="M29" s="2" t="n"/>
+      <c r="M29" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N29" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
@@ -2402,7 +2436,7 @@
       </c>
       <c r="P29" s="2" t="inlineStr">
         <is>
-          <t>Count: 2–4. Four financial signers less Party H and Party I if they were signers (likely, not stated): exactly 2 if both were. No submission reported.</t>
+          <t>Count: 6 strategic signers − Party A, Parent, Party J, Party K − 1 withdrawal (#19) = 1; met management, no submission reported in round 1.</t>
         </is>
       </c>
       <c r="Q29" s="2" t="inlineStr">
@@ -2412,7 +2446,7 @@
       </c>
       <c r="R29" s="2" t="inlineStr">
         <is>
-          <t>Q2</t>
+          <t>Q3</t>
         </is>
       </c>
       <c r="S29" s="2" t="n"/>
@@ -2430,22 +2464,22 @@
       </c>
       <c r="B30" s="2" t="inlineStr">
         <is>
-          <t>by 07/02/2021</t>
+          <t>by 06/29/2021</t>
         </is>
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Party C</t>
+          <t>2 unnamed financial signers</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Other-scope bid</t>
+          <t>Did not submit</t>
         </is>
       </c>
       <c r="F30" s="2" t="n">
@@ -2456,34 +2490,30 @@
       </c>
       <c r="H30" s="2" t="n"/>
       <c r="I30" s="2" t="n"/>
-      <c r="J30" s="2" t="inlineStr">
+      <c r="J30" s="2" t="n"/>
+      <c r="K30" s="2" t="n"/>
+      <c r="L30" s="2" t="n"/>
+      <c r="M30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="N30" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="K30" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N30" s="2" t="n"/>
-      <c r="O30" s="2" t="n"/>
+      <c r="O30" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P30" s="2" t="inlineStr">
         <is>
-          <t>Unclear: no condition stated; earlier interest was subject to further diligence. Proposes to buy a portion of the CST business for $100 million (total, not per share).</t>
+          <t>Count: 4 financial signers − Party H, Party I = 2; met management, no submission reported in round 1.</t>
         </is>
       </c>
       <c r="Q30" s="2" t="inlineStr">
         <is>
-          <t>“Party C proposed acquiring a portion of Kraton’s CST business for $100 million” (p. 35)</t>
+          <t>“By July 2, 2021, Kraton received four indications of interest as part of the first-round process that contemplated a potential acquisition of all of Kraton.” (p. 35)</t>
         </is>
       </c>
       <c r="R30" s="2" t="inlineStr">
@@ -2493,11 +2523,11 @@
       </c>
       <c r="S30" s="2" t="n"/>
       <c r="T30" s="3" t="n">
-        <v>44379</v>
+        <v>44376</v>
       </c>
       <c r="U30" s="2" t="n"/>
       <c r="V30" s="3" t="n">
-        <v>44379</v>
+        <v>44376</v>
       </c>
     </row>
     <row r="31">
@@ -2511,7 +2541,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Party G</t>
+          <t>Party J</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2521,7 +2551,7 @@
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Other-scope bid</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F31" s="2" t="n">
@@ -2532,21 +2562,9 @@
       </c>
       <c r="H31" s="2" t="n"/>
       <c r="I31" s="2" t="n"/>
-      <c r="J31" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="K31" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L31" s="2" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
+      <c r="J31" s="2" t="n"/>
+      <c r="K31" s="2" t="n"/>
+      <c r="L31" s="2" t="n"/>
       <c r="M31" s="2" t="n">
         <v>1</v>
       </c>
@@ -2554,17 +2572,17 @@
       <c r="O31" s="2" t="n"/>
       <c r="P31" s="2" t="inlineStr">
         <is>
-          <t>Unclear: subject to unspecified adjustments; earlier interest was subject to further diligence. Proposes to buy a portion of the CST business for $330 million (total, not per share).</t>
+          <t>Misses the 06/29 due date: tells J.P. Morgan it intends to submit a whole-company proposal in mid-July. Board noted this on 07/06. Party J received the process letter as a confidentiality signer.</t>
         </is>
       </c>
       <c r="Q31" s="2" t="inlineStr">
         <is>
-          <t>“Party G proposed acquiring a portion of Kraton’s CST business for $330 million, subject to adjustments.” (p. 35)</t>
+          <t>“Party J, a strategic acquirer, informed representatives of J.P. Morgan that it intended to submit a proposal to acquire Kraton during the middle of July.” (p. 35)</t>
         </is>
       </c>
       <c r="R31" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S31" s="2" t="n"/>
@@ -2587,20 +2605,20 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
+          <t>Kraton</t>
         </is>
       </c>
       <c r="D32" s="2" t="n"/>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Round opened</t>
+          <t>Deadline set</t>
         </is>
       </c>
       <c r="F32" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G32" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H32" s="2" t="n"/>
       <c r="I32" s="2" t="n"/>
@@ -2612,7 +2630,7 @@
       <c r="O32" s="2" t="n"/>
       <c r="P32" s="2" t="inlineStr">
         <is>
-          <t>Board, reviewing the four whole-company IOIs, tells Party A, Party H, Parent and Party I it requires updated IOIs ascribing greater value by 07/19 before choosing any second-round invitees. Filing prints 'July 19, 2020'; context shows 2021.</t>
+          <t>Board requires updated indications from Parties A, H, Parent and I, ascribing greater value, by 07/19 before deciding who enters the second round. Filing prints “July 19, 2020”, evidently 2021.</t>
         </is>
       </c>
       <c r="Q32" s="2" t="inlineStr">
@@ -2622,7 +2640,7 @@
       </c>
       <c r="R32" s="2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S32" s="2" t="n"/>
@@ -2664,7 +2682,7 @@
         <v>1</v>
       </c>
       <c r="G33" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H33" s="2" t="n"/>
       <c r="I33" s="2" t="n"/>
@@ -2678,17 +2696,17 @@
       <c r="O33" s="2" t="n"/>
       <c r="P33" s="2" t="inlineStr">
         <is>
-          <t>Board decides not to ask Party C, Party G or Party K for revised segment proposals 'at this time'; their proposals kept for evaluation alongside updated whole-company proposals. Not an exit.</t>
+          <t>Board decides not to ask the segment bidders for revised proposals for now; their proposals to be evaluated against the updated whole-company proposals.</t>
         </is>
       </c>
       <c r="Q33" s="2" t="inlineStr">
         <is>
-          <t>“The Board also determined not to request that Party C, Party G, or Party K submit revised indications of interest regarding their proposals to acquire portions of” (p. 35)</t>
+          <t>“The Board also determined not to request that Party C , Party G , or Party K submit revised indications of interest” (p. 35)</t>
         </is>
       </c>
       <c r="R33" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="S33" s="2" t="n"/>
@@ -2726,7 +2744,7 @@
         <v>1</v>
       </c>
       <c r="G34" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H34" s="2" t="n"/>
       <c r="I34" s="2" t="n"/>
@@ -2738,12 +2756,12 @@
       <c r="O34" s="2" t="n"/>
       <c r="P34" s="2" t="inlineStr">
         <is>
-          <t>Media report that Kraton hired J.P. Morgan for a potential sale. Ref: $31.65 close 07/02/2021 (last unaffected day); $36.37 close 07/06/2021; $34.51–$42.80 closes thereafter to signing.</t>
+          <t>Media report: Reuters says Kraton hired J.P. Morgan to advise on a potential sale. Ref: $36.37 close 07/06/2021; closes ranged $34.51–$42.80 from then to signing.</t>
         </is>
       </c>
       <c r="Q34" s="2" t="inlineStr">
         <is>
-          <t>“Reuters published a report stating, among other matters, that Kraton had hired J.P. Morgan as its financial advisor to advise Kraton with respect to a potential sale of the company” (p. 35)</t>
+          <t>“Also on July 6, 2021, Reuters published a report stating, among other matters, that Kraton had hired J.P. Morgan as its financial advisor” (p. 35)</t>
         </is>
       </c>
       <c r="R34" s="2" t="n"/>
@@ -2786,7 +2804,7 @@
         <v>1</v>
       </c>
       <c r="G35" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H35" s="2" t="n"/>
       <c r="I35" s="2" t="n"/>
@@ -2800,7 +2818,7 @@
       <c r="O35" s="2" t="n"/>
       <c r="P35" s="2" t="inlineStr">
         <is>
-          <t>Inbound inquiries to J.P. Morgan after the Reuters report; invited to sign an NDA and bid; all five declined NDAs and made no proposals, so never entered.</t>
+          <t>Inbound inquiries to J.P. Morgan about the process after the Reuters report; each invited to sign a confidentiality agreement and propose; all five declined to sign and never proposed. Never entered.</t>
         </is>
       </c>
       <c r="Q35" s="2" t="inlineStr">
@@ -2808,7 +2826,11 @@
           <t>“J.P. Morgan received inbound inquiries from six additional parties, five of which were strategic acquirers, and one of which was a financial acquirer” (p. 35)</t>
         </is>
       </c>
-      <c r="R35" s="2" t="n"/>
+      <c r="R35" s="2" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
       <c r="S35" s="2" t="n"/>
       <c r="T35" s="3" t="n">
         <v>44383</v>
@@ -2829,7 +2851,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Post-Reuters financial party</t>
+          <t>Unnamed financial party (post-Reuters)</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2846,7 +2868,7 @@
         <v>1</v>
       </c>
       <c r="G36" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H36" s="2" t="n"/>
       <c r="I36" s="2" t="n"/>
@@ -2860,15 +2882,19 @@
       <c r="O36" s="2" t="n"/>
       <c r="P36" s="2" t="inlineStr">
         <is>
-          <t>Inbound inquiry to J.P. Morgan after the Reuters report; invited to sign an NDA and submit a proposal.</t>
+          <t>Inbound inquiry after the Reuters report; invited to sign a confidentiality agreement and submit a proposal.</t>
         </is>
       </c>
       <c r="Q36" s="2" t="inlineStr">
         <is>
-          <t>“J.P. Morgan received inbound inquiries from six additional parties, five of which were strategic acquirers, and one of which was a financial acquirer” (p. 35)</t>
-        </is>
-      </c>
-      <c r="R36" s="2" t="n"/>
+          <t>“Each of these parties were invited to execute a confidentiality agreement and submit a proposal to acquire Kraton.” (p. 35)</t>
+        </is>
+      </c>
+      <c r="R36" s="2" t="inlineStr">
+        <is>
+          <t>Q5</t>
+        </is>
+      </c>
       <c r="S36" s="2" t="n"/>
       <c r="T36" s="3" t="n">
         <v>44383</v>
@@ -2889,7 +2915,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Post-Reuters financial party</t>
+          <t>Unnamed financial party (post-Reuters)</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2906,7 +2932,7 @@
         <v>1</v>
       </c>
       <c r="G37" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H37" s="2" t="n"/>
       <c r="I37" s="2" t="n"/>
@@ -2920,17 +2946,17 @@
       <c r="O37" s="2" t="n"/>
       <c r="P37" s="2" t="inlineStr">
         <is>
-          <t>Late entrant signs an NDA (11th confidentiality agreement in the process). Execution date not stated.</t>
+          <t>Eleventh confidentiality signer; also held a preliminary management meeting. Execution date not given beyond “after” 07/06.</t>
         </is>
       </c>
       <c r="Q37" s="2" t="inlineStr">
         <is>
-          <t>“Of these six parties, one party, a financial acquirer, executed a confidentiality agreement with Kraton” (p. 35)</t>
+          <t>“one party, a financial acquirer, executed a confidentiality agreement with Kraton and participated in a preliminary management meeting” (p. 35)</t>
         </is>
       </c>
       <c r="R37" s="2" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="S37" s="2" t="n"/>
@@ -2948,35 +2974,51 @@
       </c>
       <c r="B38" s="2" t="inlineStr">
         <is>
-          <t>after 07/06/2021</t>
+          <t>by 07/19/2021</t>
         </is>
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>Post-Reuters financial party</t>
+          <t>Party J</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F38" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G38" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H38" s="2" t="n"/>
-      <c r="I38" s="2" t="n"/>
-      <c r="J38" s="2" t="n"/>
-      <c r="K38" s="2" t="n"/>
-      <c r="L38" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="H38" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="I38" s="4" t="n">
+        <v>41</v>
+      </c>
+      <c r="J38" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K38" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L38" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
       <c r="M38" s="2" t="n">
         <v>1</v>
       </c>
@@ -2984,27 +3026,29 @@
       <c r="O38" s="2" t="n"/>
       <c r="P38" s="2" t="inlineStr">
         <is>
-          <t>Catch-up access: Kraton holds a preliminary management meeting with the late entrant, the access first-round NDA signers had in June. Date not stated.</t>
+          <t>Unclear: no stated conditions; first-round indication. Late whole-company indication (first price from J), received without a new due date for J; J said it would not go above this range.</t>
         </is>
       </c>
       <c r="Q38" s="2" t="inlineStr">
         <is>
-          <t>“executed a confidentiality agreement with Kraton and participated in a preliminary management meeting with Kraton’s senior” (p. 35)</t>
+          <t>“Party J also submitted an indication of interest that proposed an acquisition of Kraton at a per share purchase price of $38.00 to $41.00 per share.” (p. 36)</t>
         </is>
       </c>
       <c r="R38" s="2" t="inlineStr">
         <is>
-          <t>Q6</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S38" s="2" t="n"/>
       <c r="T38" s="3" t="n">
-        <v>44383</v>
+        <v>44389</v>
       </c>
       <c r="U38" s="3" t="n">
         <v>44383</v>
       </c>
-      <c r="V38" s="2" t="n"/>
+      <c r="V38" s="3" t="n">
+        <v>44396</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="n">
@@ -3012,55 +3056,73 @@
       </c>
       <c r="B39" s="2" t="inlineStr">
         <is>
-          <t>07/19/2021</t>
+          <t>by 07/19/2021</t>
         </is>
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
-        </is>
-      </c>
-      <c r="D39" s="2" t="n"/>
+          <t>Party A</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Deadline</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F39" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G39" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H39" s="2" t="n"/>
-      <c r="I39" s="2" t="n"/>
-      <c r="J39" s="2" t="n"/>
-      <c r="K39" s="2" t="n"/>
-      <c r="L39" s="2" t="n"/>
-      <c r="M39" s="2" t="n"/>
+        <v>1</v>
+      </c>
+      <c r="H39" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="I39" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="J39" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr">
+        <is>
+          <t>Informal</t>
+        </is>
+      </c>
+      <c r="L39" s="2" t="inlineStr">
+        <is>
+          <t>Unclear</t>
+        </is>
+      </c>
+      <c r="M39" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N39" s="2" t="n"/>
       <c r="O39" s="2" t="n"/>
       <c r="P39" s="2" t="inlineStr">
         <is>
-          <t>Due date for updated IOIs from the four whole-company bidders; responses received by 07/19/2021.</t>
+          <t>Unclear: no stated conditions; updated indication with diligence continuing. Revises #23 from $42.00–$45.00 to a point price.</t>
         </is>
       </c>
       <c r="Q39" s="2" t="inlineStr">
         <is>
-          <t>“By July 19, 2021, Kraton received updated indications of interest with respect to a potential acquisition of the entire Company” (p. 36)</t>
-        </is>
-      </c>
-      <c r="R39" s="2" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
+          <t>“Party A proposed $45.00, Party H proposed $42.00 to $45.00, and Parent proposed $45.00” (p. 36)</t>
+        </is>
+      </c>
+      <c r="R39" s="2" t="n"/>
       <c r="S39" s="2" t="n"/>
       <c r="T39" s="3" t="n">
         <v>44396</v>
       </c>
       <c r="U39" s="3" t="n">
-        <v>44396</v>
+        <v>44383</v>
       </c>
       <c r="V39" s="3" t="n">
         <v>44396</v>
@@ -3077,12 +3139,12 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>Party A</t>
+          <t>Party H</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
@@ -3094,10 +3156,10 @@
         <v>1</v>
       </c>
       <c r="G40" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H40" s="4" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I40" s="4" t="n">
         <v>45</v>
@@ -3124,12 +3186,12 @@
       <c r="O40" s="2" t="n"/>
       <c r="P40" s="2" t="inlineStr">
         <is>
-          <t>No conditions stated; second-round diligence not yet opened. Updated IOI at $45.00, up from $42.00–$45.00 (#21).</t>
+          <t>Unclear: no stated conditions; updated indication with diligence continuing. Revises #24 from $41.00–$43.00.</t>
         </is>
       </c>
       <c r="Q40" s="2" t="inlineStr">
         <is>
-          <t>“Party A proposed $45.00, Party H proposed $42.00 to $45.00, and Parent proposed $45.00.” (p. 36)</t>
+          <t>“Party A proposed $45.00, Party H proposed $42.00 to $45.00, and Parent proposed $45.00” (p. 36)</t>
         </is>
       </c>
       <c r="R40" s="2" t="n"/>
@@ -3155,12 +3217,12 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>Party H</t>
+          <t>Parent (DL Chemical Co., Ltd.)</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
@@ -3172,10 +3234,10 @@
         <v>1</v>
       </c>
       <c r="G41" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H41" s="4" t="n">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="I41" s="4" t="n">
         <v>45</v>
@@ -3202,12 +3264,12 @@
       <c r="O41" s="2" t="n"/>
       <c r="P41" s="2" t="inlineStr">
         <is>
-          <t>No conditions stated; second-round diligence not yet opened. Updated IOI at $42.00–$45.00, up from $41.00–$43.00 (#22).</t>
+          <t>Unclear: no stated conditions; updated indication with diligence continuing. Revises #25 from $41.00.</t>
         </is>
       </c>
       <c r="Q41" s="2" t="inlineStr">
         <is>
-          <t>“Party A proposed $45.00, Party H proposed $42.00 to $45.00, and Parent proposed $45.00.” (p. 36)</t>
+          <t>“Party A proposed $45.00, Party H proposed $42.00 to $45.00, and Parent proposed $45.00” (p. 36)</t>
         </is>
       </c>
       <c r="R41" s="2" t="n"/>
@@ -3233,46 +3295,30 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>Parent (DL Chemical)</t>
+          <t>Party I</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F42" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G42" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H42" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="I42" s="4" t="n">
-        <v>45</v>
-      </c>
-      <c r="J42" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="K42" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L42" s="2" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="H42" s="2" t="n"/>
+      <c r="I42" s="2" t="n"/>
+      <c r="J42" s="2" t="n"/>
+      <c r="K42" s="2" t="n"/>
+      <c r="L42" s="2" t="n"/>
       <c r="M42" s="2" t="n">
         <v>1</v>
       </c>
@@ -3280,15 +3326,19 @@
       <c r="O42" s="2" t="n"/>
       <c r="P42" s="2" t="inlineStr">
         <is>
-          <t>No conditions stated; second-round diligence not yet opened. Updated IOI at $45.00, up from $41.00 (#23).</t>
+          <t>Declines the Board's request for a higher value: will not increase its $40.00 indication (#26). No new bid.</t>
         </is>
       </c>
       <c r="Q42" s="2" t="inlineStr">
         <is>
-          <t>“Party A proposed $45.00, Party H proposed $42.00 to $45.00, and Parent proposed $45.00.” (p. 36)</t>
-        </is>
-      </c>
-      <c r="R42" s="2" t="n"/>
+          <t>“Party I stated that it was not willing to increase its proposed purchase price of $40.00 per share.” (p. 36)</t>
+        </is>
+      </c>
+      <c r="R42" s="2" t="inlineStr">
+        <is>
+          <t>Q6</t>
+        </is>
+      </c>
       <c r="S42" s="2" t="n"/>
       <c r="T42" s="3" t="n">
         <v>44396</v>
@@ -3306,53 +3356,47 @@
       </c>
       <c r="B43" s="2" t="inlineStr">
         <is>
-          <t>by 07/19/2021</t>
+          <t>07/19/2021</t>
         </is>
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>Party I</t>
-        </is>
-      </c>
-      <c r="D43" s="2" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
+          <t>Kraton</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="n"/>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Deadline</t>
         </is>
       </c>
       <c r="F43" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G43" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H43" s="2" t="n"/>
       <c r="I43" s="2" t="n"/>
       <c r="J43" s="2" t="n"/>
       <c r="K43" s="2" t="n"/>
       <c r="L43" s="2" t="n"/>
-      <c r="M43" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="M43" s="2" t="n"/>
       <c r="N43" s="2" t="n"/>
       <c r="O43" s="2" t="n"/>
       <c r="P43" s="2" t="inlineStr">
         <is>
-          <t>Party I answers the request for greater value by refusing to raise its $40.00 (#24); no new bid.</t>
+          <t>Due date for updated indications from A, H, Parent and I; all four responded by it. Board acted on the bids in hand on 07/20.</t>
         </is>
       </c>
       <c r="Q43" s="2" t="inlineStr">
         <is>
-          <t>“Party I stated that it was not willing to increase its proposed purchase price of $40.00 per share.” (p. 36)</t>
+          <t>“By July 19, 2021, Kraton received updated indications of interest with respect to a potential acquisition of the entire Company” (p. 36)</t>
         </is>
       </c>
       <c r="R43" s="2" t="inlineStr">
         <is>
-          <t>Q7</t>
+          <t>Q4</t>
         </is>
       </c>
       <c r="S43" s="2" t="n"/>
@@ -3360,7 +3404,7 @@
         <v>44396</v>
       </c>
       <c r="U43" s="3" t="n">
-        <v>44383</v>
+        <v>44396</v>
       </c>
       <c r="V43" s="3" t="n">
         <v>44396</v>
@@ -3372,29 +3416,29 @@
       </c>
       <c r="B44" s="2" t="inlineStr">
         <is>
-          <t>by 07/19/2021</t>
+          <t>07/20/2021</t>
         </is>
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>Party J</t>
+          <t>Party I</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
         <is>
-          <t>Strategic</t>
+          <t>Financial</t>
         </is>
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Re-entered</t>
+          <t>Dropped by target</t>
         </is>
       </c>
       <c r="F44" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G44" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H44" s="2" t="n"/>
       <c r="I44" s="2" t="n"/>
@@ -3404,30 +3448,40 @@
       <c r="M44" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N44" s="2" t="n"/>
-      <c r="O44" s="2" t="n"/>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>Would not improve earlier offer</t>
+        </is>
+      </c>
+      <c r="O44" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P44" s="2" t="inlineStr">
         <is>
-          <t>Party J returns after not submitting in round 1 (#25), with its announced mid-July bid; not among the four asked for updated IOIs, so received but not admitted.</t>
+          <t>Not among the three invited to round 2 (complete set named), after refusing to raise its $40.00 indication when asked (#41).</t>
         </is>
       </c>
       <c r="Q44" s="2" t="inlineStr">
         <is>
-          <t>“Party J also submitted an indication of interest that proposed an acquisition of Kraton at a per share purchase price of $38.00 to $41.00 per share.” (p. 36)</t>
+          <t>“invite Party A , Party H, and Parent to the second round of the transaction process” (p. 36)</t>
         </is>
       </c>
       <c r="R44" s="2" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="S44" s="2" t="n"/>
       <c r="T44" s="3" t="n">
-        <v>44396</v>
-      </c>
-      <c r="U44" s="2" t="n"/>
+        <v>44397</v>
+      </c>
+      <c r="U44" s="3" t="n">
+        <v>44397</v>
+      </c>
       <c r="V44" s="3" t="n">
-        <v>44396</v>
+        <v>44397</v>
       </c>
     </row>
     <row r="45">
@@ -3436,7 +3490,7 @@
       </c>
       <c r="B45" s="2" t="inlineStr">
         <is>
-          <t>by 07/19/2021</t>
+          <t>07/20/2021</t>
         </is>
       </c>
       <c r="C45" s="2" t="inlineStr">
@@ -3451,63 +3505,57 @@
       </c>
       <c r="E45" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Dropped by target</t>
         </is>
       </c>
       <c r="F45" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G45" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H45" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="I45" s="4" t="n">
-        <v>41</v>
-      </c>
-      <c r="J45" s="2" t="inlineStr">
+        <v>1</v>
+      </c>
+      <c r="H45" s="2" t="n"/>
+      <c r="I45" s="2" t="n"/>
+      <c r="J45" s="2" t="n"/>
+      <c r="K45" s="2" t="n"/>
+      <c r="L45" s="2" t="n"/>
+      <c r="M45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N45" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
         </is>
       </c>
-      <c r="K45" s="2" t="inlineStr">
-        <is>
-          <t>Informal</t>
-        </is>
-      </c>
-      <c r="L45" s="2" t="inlineStr">
-        <is>
-          <t>Unclear</t>
-        </is>
-      </c>
-      <c r="M45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N45" s="2" t="n"/>
-      <c r="O45" s="2" t="n"/>
+      <c r="O45" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P45" s="2" t="inlineStr">
         <is>
-          <t>No conditions stated; diligence open. First IOI, $38.00–$41.00, and J said it would not go above this range. Unsolicited in round 2.</t>
+          <t>Not among the three invited to round 2 (complete set named). J had bid $38.00–$41.00 and said it would not go higher; it was not asked to improve, so no reason is attributed.</t>
         </is>
       </c>
       <c r="Q45" s="2" t="inlineStr">
         <is>
-          <t>“Party J also submitted an indication of interest that proposed an acquisition of Kraton at a per share purchase price of $38.00 to $41.00 per share.” (p. 36)</t>
+          <t>“invite Party A , Party H, and Parent to the second round of the transaction process” (p. 36)</t>
         </is>
       </c>
       <c r="R45" s="2" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q6</t>
         </is>
       </c>
       <c r="S45" s="2" t="n"/>
       <c r="T45" s="3" t="n">
-        <v>44396</v>
-      </c>
-      <c r="U45" s="2" t="n"/>
+        <v>44397</v>
+      </c>
+      <c r="U45" s="3" t="n">
+        <v>44397</v>
+      </c>
       <c r="V45" s="3" t="n">
-        <v>44396</v>
+        <v>44397</v>
       </c>
     </row>
     <row r="46">
@@ -3516,47 +3564,61 @@
       </c>
       <c r="B46" s="2" t="inlineStr">
         <is>
-          <t>07/20/2021</t>
+          <t>after 07/06/2021; by 09/27/2021</t>
         </is>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
-        </is>
-      </c>
-      <c r="D46" s="2" t="n"/>
+          <t>Unnamed financial party (post-Reuters)</t>
+        </is>
+      </c>
+      <c r="D46" s="2" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Round opened</t>
+          <t>Did not submit</t>
         </is>
       </c>
       <c r="F46" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G46" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="H46" s="2" t="n"/>
       <c r="I46" s="2" t="n"/>
       <c r="J46" s="2" t="n"/>
       <c r="K46" s="2" t="n"/>
       <c r="L46" s="2" t="n"/>
-      <c r="M46" s="2" t="n"/>
-      <c r="N46" s="2" t="n"/>
-      <c r="O46" s="2" t="n"/>
+      <c r="M46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N46" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="O46" s="2" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
       <c r="P46" s="2" t="inlineStr">
         <is>
-          <t>Board selects Party A, Party H and Parent for the filing's 'second round' and gives all three additional financial and diligence materials; diligence management meetings week of 08/09/2021. No bid due date yet. Board also asks for analysis of separate segment sales.</t>
+          <t>Filing reports it never submitted a proposal after being invited to; timing inferred. Sorted at the 07/20 advancement decision, which named a complete set without it.</t>
         </is>
       </c>
       <c r="Q46" s="2" t="inlineStr">
         <is>
-          <t>“the Board instructed representatives of J.P. Morgan and Kraton’s senior management to invite Party A, Party H, and Parent to the second round of the transaction process” (p. 36)</t>
+          <t>“management but did not submit any proposal with respect to a transaction.” (p. 36)</t>
         </is>
       </c>
       <c r="R46" s="2" t="inlineStr">
         <is>
-          <t>Q1</t>
+          <t>Q5</t>
         </is>
       </c>
       <c r="S46" s="2" t="n"/>
@@ -3564,10 +3626,10 @@
         <v>44397</v>
       </c>
       <c r="U46" s="3" t="n">
-        <v>44397</v>
+        <v>44383</v>
       </c>
       <c r="V46" s="3" t="n">
-        <v>44397</v>
+        <v>44466</v>
       </c>
     </row>
     <row r="47">
@@ -3581,17 +3643,13 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Party I</t>
-        </is>
-      </c>
-      <c r="D47" s="2" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
+          <t>Kraton</t>
+        </is>
+      </c>
+      <c r="D47" s="2" t="n"/>
       <c r="E47" s="2" t="inlineStr">
         <is>
-          <t>Dropped by target</t>
+          <t>Round opened</t>
         </is>
       </c>
       <c r="F47" s="2" t="n">
@@ -3605,32 +3663,22 @@
       <c r="J47" s="2" t="n"/>
       <c r="K47" s="2" t="n"/>
       <c r="L47" s="2" t="n"/>
-      <c r="M47" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N47" s="2" t="inlineStr">
-        <is>
-          <t>Would not improve earlier offer</t>
-        </is>
-      </c>
-      <c r="O47" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M47" s="2" t="n"/>
+      <c r="N47" s="2" t="n"/>
+      <c r="O47" s="2" t="n"/>
       <c r="P47" s="2" t="inlineStr">
         <is>
-          <t>Not in the named advancing set (#45). Party I had been asked for greater value and refused to raise $40.00 (#42).</t>
+          <t>Board advances Parties A and H and Parent, to receive additional financial and diligence materials (alike for all three); diligence management meetings week of 08/09. No bid requested. Board also asks J.P. Morgan to analyse separate segment sales.</t>
         </is>
       </c>
       <c r="Q47" s="2" t="inlineStr">
         <is>
-          <t>“the Board instructed representatives of J.P. Morgan and Kraton’s senior management to invite Party A, Party H, and Parent to the second round of the transaction process” (p. 36)</t>
+          <t>“the Board instructed representatives of J.P. Morgan and Kraton’s senior management to invite Party A , Party H, and Parent to the second round of the transaction process” (p. 36)</t>
         </is>
       </c>
       <c r="R47" s="2" t="inlineStr">
         <is>
-          <t>Q7</t>
+          <t>Q2</t>
         </is>
       </c>
       <c r="S47" s="2" t="n"/>
@@ -3650,12 +3698,12 @@
       </c>
       <c r="B48" s="2" t="inlineStr">
         <is>
-          <t>07/20/2021</t>
+          <t>08/04/2021</t>
         </is>
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Party J</t>
+          <t>Party G</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -3665,7 +3713,7 @@
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Dropped by target</t>
+          <t>Withdrew</t>
         </is>
       </c>
       <c r="F48" s="2" t="n">
@@ -3687,35 +3735,31 @@
           <t>Not stated</t>
         </is>
       </c>
-      <c r="O48" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="O48" s="2" t="n"/>
       <c r="P48" s="2" t="inlineStr">
         <is>
-          <t>Not in the named advancing set (#45); its $38.00–$41.00 was below the other three bids. J was not asked to improve.</t>
+          <t>Segment-only participant: no longer interested in the CST business; its $330 million proposal (#10) lapses.</t>
         </is>
       </c>
       <c r="Q48" s="2" t="inlineStr">
         <is>
-          <t>“the Board instructed representatives of J.P. Morgan and Kraton’s senior management to invite Party A, Party H, and Parent to the second round of the transaction process” (p. 36)</t>
+          <t>“On August 4, 2021, Party G informed Kraton that it was no longer interested in acquiring Kraton’s CST business.” (p. 36)</t>
         </is>
       </c>
       <c r="R48" s="2" t="inlineStr">
         <is>
-          <t>Q5</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="S48" s="2" t="n"/>
       <c r="T48" s="3" t="n">
-        <v>44397</v>
+        <v>44412</v>
       </c>
       <c r="U48" s="3" t="n">
-        <v>44397</v>
+        <v>44412</v>
       </c>
       <c r="V48" s="3" t="n">
-        <v>44397</v>
+        <v>44412</v>
       </c>
     </row>
     <row r="49">
@@ -3724,22 +3768,18 @@
       </c>
       <c r="B49" s="2" t="inlineStr">
         <is>
-          <t>08/04/2021</t>
+          <t>after 08/11/2021</t>
         </is>
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Party G</t>
-        </is>
-      </c>
-      <c r="D49" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Kraton</t>
+        </is>
+      </c>
+      <c r="D49" s="2" t="n"/>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Withdrew</t>
+          <t>Round opened</t>
         </is>
       </c>
       <c r="F49" s="2" t="n">
@@ -3753,39 +3793,33 @@
       <c r="J49" s="2" t="n"/>
       <c r="K49" s="2" t="n"/>
       <c r="L49" s="2" t="n"/>
-      <c r="M49" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N49" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
+      <c r="M49" s="2" t="n"/>
+      <c r="N49" s="2" t="n"/>
       <c r="O49" s="2" t="n"/>
       <c r="P49" s="2" t="inlineStr">
         <is>
-          <t>CST-only bidder (#30): no longer interested in acquiring the CST business.</t>
+          <t>Final bid procedures letter to Parties A and H and Parent: merger agreement markups due 09/08, final indications due 09/15. Sent after the 08/11 Board meeting authorized the draft merger agreement; sorted at that decision.</t>
         </is>
       </c>
       <c r="Q49" s="2" t="inlineStr">
         <is>
-          <t>“On August 4, 2021, Party G informed Kraton that it was no longer interested in acquiring Kraton’s CST business.” (p. 36)</t>
+          <t>“J.P. Morgan provided a final bid procedures letter to Party A , Party H, and Parent that requested these bidders to submit markups of a draft merger agreement” (p. 37)</t>
         </is>
       </c>
       <c r="R49" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q2; Q7</t>
         </is>
       </c>
       <c r="S49" s="2" t="n"/>
       <c r="T49" s="3" t="n">
-        <v>44412</v>
+        <v>44419</v>
       </c>
       <c r="U49" s="3" t="n">
-        <v>44412</v>
+        <v>44419</v>
       </c>
       <c r="V49" s="3" t="n">
-        <v>44412</v>
+        <v>44446</v>
       </c>
     </row>
     <row r="50">
@@ -3799,7 +3833,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Media outlet 1</t>
+          <t>Media outlet</t>
         </is>
       </c>
       <c r="D50" s="2" t="n"/>
@@ -3824,7 +3858,7 @@
       <c r="O50" s="2" t="n"/>
       <c r="P50" s="2" t="inlineStr">
         <is>
-          <t>Media report that potential acquirers had been invited to a second round.</t>
+          <t>Media report that potential acquirers had been invited to a second round (first of two outlets).</t>
         </is>
       </c>
       <c r="Q50" s="2" t="inlineStr">
@@ -3850,25 +3884,25 @@
       </c>
       <c r="B51" s="2" t="inlineStr">
         <is>
-          <t>after 08/11/2021, by 08/20/2021</t>
+          <t>08/16/2021</t>
         </is>
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
+          <t>Media outlet</t>
         </is>
       </c>
       <c r="D51" s="2" t="n"/>
       <c r="E51" s="2" t="inlineStr">
         <is>
-          <t>Round opened</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F51" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G51" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H51" s="2" t="n"/>
       <c r="I51" s="2" t="n"/>
@@ -3880,28 +3914,24 @@
       <c r="O51" s="2" t="n"/>
       <c r="P51" s="2" t="inlineStr">
         <is>
-          <t>Final bid procedures letter to Party A, Party H and Parent: merger agreement markups due 09/08/2021, final IOIs due 09/15/2021; Board authorized sending the draft merger agreement 08/11. Date to 08/20 inferred: Party H received the letter and quit that day.</t>
+          <t>Second media report that potential acquirers had been invited to a second round.</t>
         </is>
       </c>
       <c r="Q51" s="2" t="inlineStr">
         <is>
-          <t>“a final bid procedures letter to Party A, Party H, and Parent that requested these bidders to submit markups of a draft merger agreement by September 8, 2021” (p. 37)</t>
-        </is>
-      </c>
-      <c r="R51" s="2" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
-      </c>
+          <t>“On August 13 and August 16, 2021, two media outlets each published a report stating, among other matters, that potential acquirers of Kraton had been invited to the second round” (p. 37)</t>
+        </is>
+      </c>
+      <c r="R51" s="2" t="n"/>
       <c r="S51" s="2" t="n"/>
       <c r="T51" s="3" t="n">
-        <v>44423</v>
+        <v>44424</v>
       </c>
       <c r="U51" s="3" t="n">
-        <v>44419</v>
+        <v>44424</v>
       </c>
       <c r="V51" s="3" t="n">
-        <v>44428</v>
+        <v>44424</v>
       </c>
     </row>
     <row r="52">
@@ -3910,54 +3940,64 @@
       </c>
       <c r="B52" s="2" t="inlineStr">
         <is>
-          <t>08/16/2021</t>
+          <t>08/20/2021</t>
         </is>
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Media outlet 2</t>
-        </is>
-      </c>
-      <c r="D52" s="2" t="n"/>
+          <t>Party H</t>
+        </is>
+      </c>
+      <c r="D52" s="2" t="inlineStr">
+        <is>
+          <t>Financial</t>
+        </is>
+      </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Withdrew</t>
         </is>
       </c>
       <c r="F52" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G52" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H52" s="2" t="n"/>
       <c r="I52" s="2" t="n"/>
       <c r="J52" s="2" t="n"/>
       <c r="K52" s="2" t="n"/>
       <c r="L52" s="2" t="n"/>
-      <c r="M52" s="2" t="n"/>
-      <c r="N52" s="2" t="n"/>
+      <c r="M52" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="N52" s="2" t="inlineStr">
+        <is>
+          <t>Value below earlier offer</t>
+        </is>
+      </c>
       <c r="O52" s="2" t="n"/>
       <c r="P52" s="2" t="inlineStr">
         <is>
-          <t>Second media report that potential acquirers had been invited to a second round.</t>
+          <t>Tells Kraton it cannot maintain its $42.00–$45.00 indicative range (#39) and cannot continue in the process.</t>
         </is>
       </c>
       <c r="Q52" s="2" t="inlineStr">
         <is>
-          <t>“On August 13 and August 16, 2021, two media outlets each published a report stating, among other matters, that potential acquirers of Kraton had been invited to the second round” (p. 37)</t>
+          <t>“On August 20, 2021, Party H informed Kraton that it was unable to maintain its indicative bid price range and was unable to continue in the process.” (p. 37)</t>
         </is>
       </c>
       <c r="R52" s="2" t="n"/>
       <c r="S52" s="2" t="n"/>
       <c r="T52" s="3" t="n">
-        <v>44424</v>
+        <v>44428</v>
       </c>
       <c r="U52" s="3" t="n">
-        <v>44424</v>
+        <v>44428</v>
       </c>
       <c r="V52" s="3" t="n">
-        <v>44424</v>
+        <v>44428</v>
       </c>
     </row>
     <row r="53">
@@ -3966,29 +4006,29 @@
       </c>
       <c r="B53" s="2" t="inlineStr">
         <is>
-          <t>08/20/2021</t>
+          <t>08/30/2021</t>
         </is>
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Party H</t>
+          <t>Party K</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
         <is>
-          <t>Financial</t>
+          <t>Strategic</t>
         </is>
       </c>
       <c r="E53" s="2" t="inlineStr">
         <is>
-          <t>Withdrew</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F53" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G53" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H53" s="2" t="n"/>
       <c r="I53" s="2" t="n"/>
@@ -3998,32 +4038,32 @@
       <c r="M53" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="N53" s="2" t="inlineStr">
-        <is>
-          <t>Value below earlier offer</t>
-        </is>
-      </c>
+      <c r="N53" s="2" t="n"/>
       <c r="O53" s="2" t="n"/>
       <c r="P53" s="2" t="inlineStr">
         <is>
-          <t>Party H said it could not maintain its $42.00–$45.00 indicative range (#40) and could not continue, implying value below its earlier offer.</t>
+          <t>Board, finding a sum-of-the-parts sale unlikely to beat a whole-company sale, asks J.P. Morgan to request an updated chemical-segment proposal from K. J.P. Morgan noted K's proposal needed significant diligence and firm financing; Party C's $100 million CST bid was the only other live chemical proposal.</t>
         </is>
       </c>
       <c r="Q53" s="2" t="inlineStr">
         <is>
-          <t>“Party H informed Kraton that it was unable to maintain its indicative bid price range and was unable to continue in the process.” (p. 37)</t>
-        </is>
-      </c>
-      <c r="R53" s="2" t="n"/>
+          <t>“the Board therefore instructed J.P. Morgan to request an updated proposal from Party K regarding its possible acquisition of Kraton’s chemical segment” (p. 38)</t>
+        </is>
+      </c>
+      <c r="R53" s="2" t="inlineStr">
+        <is>
+          <t>Q1</t>
+        </is>
+      </c>
       <c r="S53" s="2" t="n"/>
       <c r="T53" s="3" t="n">
-        <v>44428</v>
+        <v>44438</v>
       </c>
       <c r="U53" s="3" t="n">
-        <v>44428</v>
+        <v>44438</v>
       </c>
       <c r="V53" s="3" t="n">
-        <v>44428</v>
+        <v>44438</v>
       </c>
     </row>
     <row r="54">
@@ -4032,25 +4072,25 @@
       </c>
       <c r="B54" s="2" t="inlineStr">
         <is>
-          <t>08/30/2021</t>
+          <t>09/08/2021</t>
         </is>
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
+          <t>Kraton</t>
         </is>
       </c>
       <c r="D54" s="2" t="n"/>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Other material event</t>
+          <t>Deadline</t>
         </is>
       </c>
       <c r="F54" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G54" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H54" s="2" t="n"/>
       <c r="I54" s="2" t="n"/>
@@ -4062,24 +4102,28 @@
       <c r="O54" s="2" t="n"/>
       <c r="P54" s="2" t="inlineStr">
         <is>
-          <t>After 08/22 and 08/30 Sum of the Parts reviews, Board finds separate segment sales unlikely to beat a whole-company sale but keeps alternatives open; asks J.P. Morgan to request an updated proposal from Party K.</t>
+          <t>Due date for merger agreement markups; Parent and Party A both delivered on the day. Bidding continued to the 09/15 due date.</t>
         </is>
       </c>
       <c r="Q54" s="2" t="inlineStr">
         <is>
-          <t>“the Board therefore instructed J.P. Morgan to request an updated proposal from Party K regarding its possible acquisition of Kraton’s chemical segment” (p. 38)</t>
-        </is>
-      </c>
-      <c r="R54" s="2" t="n"/>
+          <t>“On September 8, 2021, Parent and Party A submitted their markups of the draft merger agreement.” (p. 38)</t>
+        </is>
+      </c>
+      <c r="R54" s="2" t="inlineStr">
+        <is>
+          <t>Q7</t>
+        </is>
+      </c>
       <c r="S54" s="2" t="n"/>
       <c r="T54" s="3" t="n">
-        <v>44438</v>
+        <v>44447</v>
       </c>
       <c r="U54" s="3" t="n">
-        <v>44438</v>
+        <v>44447</v>
       </c>
       <c r="V54" s="3" t="n">
-        <v>44438</v>
+        <v>44447</v>
       </c>
     </row>
     <row r="55">
@@ -4093,7 +4137,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Parent (DL Chemical)</t>
+          <t>Parent (DL Chemical Co., Ltd.)</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -4110,7 +4154,7 @@
         <v>1</v>
       </c>
       <c r="G55" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H55" s="2" t="n"/>
       <c r="I55" s="2" t="n"/>
@@ -4124,12 +4168,12 @@
       <c r="O55" s="2" t="n"/>
       <c r="P55" s="2" t="inlineStr">
         <is>
-          <t>Parent submits merger agreement markup, no new price: deletes hell-or-high-water; company termination fee 3.5% of enterprise value (vs 2% equity); no financing condition, but delayed debt marketing period and specific performance/damages as sole recourse on financing failure.</t>
+          <t>Submits merger agreement markup supporting its $45.00 indication (#40): deletes hell-or-high-water, seeks 3.5% of enterprise value company fee (vs 2% of equity), no financing condition but debt marketing period and specific performance/damages as Kraton's only recourse on financing failure.</t>
         </is>
       </c>
       <c r="Q55" s="2" t="inlineStr">
         <is>
-          <t>“On September 8, 2021, Parent and Party A submitted their markups of the draft merger agreement.” (p. 38)</t>
+          <t>“Parent’s markup deleted the “hell or high water” regulatory provisions included in the Company’s draft merger agreement” (p. 38)</t>
         </is>
       </c>
       <c r="R55" s="2" t="inlineStr">
@@ -4176,7 +4220,7 @@
         <v>1</v>
       </c>
       <c r="G56" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H56" s="2" t="n"/>
       <c r="I56" s="2" t="n"/>
@@ -4190,7 +4234,7 @@
       <c r="O56" s="2" t="n"/>
       <c r="P56" s="2" t="inlineStr">
         <is>
-          <t>Party A submits its merger agreement markup on the markup due date, no new price; contents not described.</t>
+          <t>Submits its merger agreement markup, supporting its $45.00 indication (#38); terms of the markup not described.</t>
         </is>
       </c>
       <c r="Q56" s="2" t="inlineStr">
@@ -4242,7 +4286,7 @@
         <v>1</v>
       </c>
       <c r="G57" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H57" s="2" t="n"/>
       <c r="I57" s="2" t="n"/>
@@ -4268,7 +4312,7 @@
       <c r="O57" s="2" t="n"/>
       <c r="P57" s="2" t="inlineStr">
         <is>
-          <t>Heavy: subject to further diligence and price adjustments; no debt financing talks and no equity financing arrangements. Requested update (#53): chemical segment at 9.5x trailing-12-month (Sept 2021) segment adjusted EBITDA, purported enterprise value $1.25 billion.</t>
+          <t>Heavy: subject to further diligence and price adjustments; no debt financing discussions and no equity financing arranged. Chemical segment at 9.5x adjusted EBITDA for the 12 months to September 2021, which K put at about $1.25 billion enterprise value. Revises #27.</t>
         </is>
       </c>
       <c r="Q57" s="2" t="inlineStr">
@@ -4278,7 +4322,7 @@
       </c>
       <c r="R57" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="S57" s="2" t="n"/>
@@ -4303,42 +4347,64 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>Kraton (target)</t>
-        </is>
-      </c>
-      <c r="D58" s="2" t="n"/>
+          <t>Parent (DL Chemical Co., Ltd.)</t>
+        </is>
+      </c>
+      <c r="D58" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Deadline</t>
+          <t>Bid</t>
         </is>
       </c>
       <c r="F58" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G58" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H58" s="2" t="n"/>
-      <c r="I58" s="2" t="n"/>
-      <c r="J58" s="2" t="n"/>
-      <c r="K58" s="2" t="n"/>
-      <c r="L58" s="2" t="n"/>
-      <c r="M58" s="2" t="n"/>
+        <v>3</v>
+      </c>
+      <c r="H58" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="I58" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="J58" s="2" t="inlineStr">
+        <is>
+          <t>Not stated</t>
+        </is>
+      </c>
+      <c r="K58" s="2" t="inlineStr">
+        <is>
+          <t>Formal</t>
+        </is>
+      </c>
+      <c r="L58" s="2" t="inlineStr">
+        <is>
+          <t>Light</t>
+        </is>
+      </c>
+      <c r="M58" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N58" s="2" t="n"/>
       <c r="O58" s="2" t="n"/>
       <c r="P58" s="2" t="inlineStr">
         <is>
-          <t>Due date for final indications of interest (markups were due 09/08/2021). Parent bid on the day; Party A bid on 09/17/2021 and the Board reviewed it 09/18/2021.</t>
+          <t>Light: Parent said it had completed substantially all diligence; financing not a condition in its markup, no commitment yet reported. Formal: final-round bid backed by its 09/08 markup (#54). Revises #40.</t>
         </is>
       </c>
       <c r="Q58" s="2" t="inlineStr">
         <is>
-          <t>“and final indications of interest by September 15, 2021” (p. 37)</t>
+          <t>“On September 15, 2021, Parent provided a revised proposal to acquire Kraton for $46.00 per share. Parent noted that it had completed substantially all due diligence.” (p. 39)</t>
         </is>
       </c>
       <c r="R58" s="2" t="inlineStr">
         <is>
-          <t>Q4</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="S58" s="2" t="n"/>
@@ -4363,64 +4429,42 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>Parent (DL Chemical)</t>
-        </is>
-      </c>
-      <c r="D59" s="2" t="inlineStr">
-        <is>
-          <t>Strategic</t>
-        </is>
-      </c>
+          <t>Kraton</t>
+        </is>
+      </c>
+      <c r="D59" s="2" t="n"/>
       <c r="E59" s="2" t="inlineStr">
         <is>
-          <t>Bid</t>
+          <t>Deadline</t>
         </is>
       </c>
       <c r="F59" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G59" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="H59" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="I59" s="4" t="n">
-        <v>46</v>
-      </c>
-      <c r="J59" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="K59" s="2" t="inlineStr">
-        <is>
-          <t>Formal</t>
-        </is>
-      </c>
-      <c r="L59" s="2" t="inlineStr">
-        <is>
-          <t>Light</t>
-        </is>
-      </c>
-      <c r="M59" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>3</v>
+      </c>
+      <c r="H59" s="2" t="n"/>
+      <c r="I59" s="2" t="n"/>
+      <c r="J59" s="2" t="n"/>
+      <c r="K59" s="2" t="n"/>
+      <c r="L59" s="2" t="n"/>
+      <c r="M59" s="2" t="n"/>
       <c r="N59" s="2" t="n"/>
       <c r="O59" s="2" t="n"/>
       <c r="P59" s="2" t="inlineStr">
         <is>
-          <t>Light: Parent says it has completed substantially all due diligence; financing not a condition (markup #54). Formal: markup plus response to final-bid letter. $46.00 per share, up from $45.00 (#41).</t>
+          <t>Due date for final indications. Parent bid on the day; Party A bid two days late (#59) and the Board considered it on 09/18.</t>
         </is>
       </c>
       <c r="Q59" s="2" t="inlineStr">
         <is>
-          <t>“On September 15, 2021, Parent provided a revised proposal to acquire Kraton for $46.00 per share. Parent noted that it had completed substantially all due diligence.” (p. 39)</t>
+          <t>“final indications of interest by September 15, 2021” (p. 37)</t>
         </is>
       </c>
       <c r="R59" s="2" t="inlineStr">
         <is>
-          <t>Q8</t>
+          <t>Q7</t>
         </is>
       </c>
       <c r="S59" s="2" t="n"/>
@@ -4462,7 +4506,7 @@
         <v>1</v>
       </c>
       <c r="G60" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H60" s="4" t="n">
         <v>40.5</v>
@@ -4492,7 +4536,7 @@
       <c r="O60" s="2" t="n"/>
       <c r="P60" s="2" t="inlineStr">
         <is>
-          <t>Heavy: 'subject to additional due diligence'. Formal: markup (#55) plus final-round response, two days after the 09/15 due date. $40.50 per share, down from $45.00 (#39).</t>
+          <t>Heavy: subject to additional due diligence. Formal: final-round bid backed by its 09/08 markup (#55), two days after the due date. Revises #38 downward from $45.00.</t>
         </is>
       </c>
       <c r="Q60" s="2" t="inlineStr">
@@ -4502,7 +4546,7 @@
       </c>
       <c r="R60" s="2" t="inlineStr">
         <is>
-          <t>Q4; Q9</t>
+          <t>Q7; Q8</t>
         </is>
       </c>
       <c r="S60" s="2" t="n"/>
@@ -4544,7 +4588,7 @@
         <v>1</v>
       </c>
       <c r="G61" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H61" s="2" t="n"/>
       <c r="I61" s="2" t="n"/>
@@ -4570,7 +4614,7 @@
       <c r="O61" s="2" t="n"/>
       <c r="P61" s="2" t="inlineStr">
         <is>
-          <t>Heavy: subject to additional due diligence and adjustments. Alternative to #59: buys the polymer segment at $1.3 billion enterprise value while the chemical business is spun off to Kraton stockholders.</t>
+          <t>Heavy: subject to additional due diligence and adjustments. Alternative to #59: buy the polymer segment for $1.3 billion enterprise value, with the chemical business spun off to Kraton stockholders. No per-share price.</t>
         </is>
       </c>
       <c r="Q61" s="2" t="inlineStr">
@@ -4578,7 +4622,11 @@
           <t>“Party A also proposed an alternative transaction whereby it would acquire Kraton’s polymer segment for an enterprise value equal to $1.3 billion, subject to certain adjustments” (p. 39)</t>
         </is>
       </c>
-      <c r="R61" s="2" t="n"/>
+      <c r="R61" s="2" t="inlineStr">
+        <is>
+          <t>Q1; Q8</t>
+        </is>
+      </c>
       <c r="S61" s="2" t="n"/>
       <c r="T61" s="3" t="n">
         <v>44456</v>
@@ -4601,7 +4649,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>Parent (DL Chemical)</t>
+          <t>Parent (DL Chemical Co., Ltd.)</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -4618,7 +4666,7 @@
         <v>1</v>
       </c>
       <c r="G62" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H62" s="2" t="n"/>
       <c r="I62" s="2" t="n"/>
@@ -4632,12 +4680,12 @@
       <c r="O62" s="2" t="n"/>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t>Price requirement: Board asks Parent to raise to $46.50 and says Kraton expects a reverse break fee on debt financing failure. Board again rejects Sum of the Parts (updated best case about $46–$48 per share).</t>
+          <t>Price requirement: Board tells J.P. Morgan to ask Parent to raise to $46.50 and to say Kraton expects a reverse break fee on a debt financing failure. Board again rejects a sum-of-the-parts sale (best case about $46–$48).</t>
         </is>
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t>“the Board instructed J.P. Morgan to request that Parent increase its proposal to $46.50 per share, and to also inform Party A that its proposal did not provide adequate value” (p. 39)</t>
+          <t>“the Board instructed J.P. Morgan to request that Parent increase its proposal to $46.50 per share” (p. 39)</t>
         </is>
       </c>
       <c r="R62" s="2" t="n"/>
@@ -4680,7 +4728,7 @@
         <v>1</v>
       </c>
       <c r="G63" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H63" s="2" t="n"/>
       <c r="I63" s="2" t="n"/>
@@ -4694,12 +4742,12 @@
       <c r="O63" s="2" t="n"/>
       <c r="P63" s="2" t="inlineStr">
         <is>
-          <t>Board tells Party A its $40.50 proposal (#59) does not offer adequate value; Party A stays in.</t>
+          <t>Board tells J.P. Morgan to inform Party A that its proposals (#59, #60) do not provide adequate value. Party A stays in and bids again.</t>
         </is>
       </c>
       <c r="Q63" s="2" t="inlineStr">
         <is>
-          <t>“and to also inform Party A that its proposal did not provide adequate value to Kraton and its stockholders.” (p. 39)</t>
+          <t>“to also inform Party A that its proposal did not provide adequate value to Kraton and its stockholders” (p. 39)</t>
         </is>
       </c>
       <c r="R63" s="2" t="n"/>
@@ -4725,7 +4773,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>Parent (DL Chemical)</t>
+          <t>Parent (DL Chemical Co., Ltd.)</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -4742,7 +4790,7 @@
         <v>1</v>
       </c>
       <c r="G64" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H64" s="4" t="n">
         <v>46.5</v>
@@ -4772,7 +4820,7 @@
       <c r="O64" s="2" t="n"/>
       <c r="P64" s="2" t="inlineStr">
         <is>
-          <t>Light: diligence substantially complete (#58); only final documentation remained, negotiated 09/20–09/26 (termination fees settled at $63 million each way). Formal. Raises to the requested $46.50 per share, stated as best and final.</t>
+          <t>Light: diligence substantially complete (#57); debt commitment letter still in draft. Meets the Board's $46.50 request; stated as best and final. Formal. Kraton then sends a revised draft agreement to Parent's counsel; fees negotiated to 09/26.</t>
         </is>
       </c>
       <c r="Q64" s="2" t="inlineStr">
@@ -4780,7 +4828,11 @@
           <t>“Parent would increase its purchase price to $46.50 per share, and that this proposal was its best and final offer.” (p. 39)</t>
         </is>
       </c>
-      <c r="R64" s="2" t="n"/>
+      <c r="R64" s="2" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
       <c r="S64" s="2" t="n"/>
       <c r="T64" s="3" t="n">
         <v>44459</v>
@@ -4803,7 +4855,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>O’Melveny &amp; Myers LLP (Parent)</t>
+          <t>O’Melveny &amp; Myers LLP</t>
         </is>
       </c>
       <c r="D65" s="2" t="n"/>
@@ -4816,7 +4868,7 @@
         <v>1</v>
       </c>
       <c r="G65" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H65" s="2" t="n"/>
       <c r="I65" s="2" t="n"/>
@@ -4828,12 +4880,12 @@
       <c r="O65" s="2" t="n"/>
       <c r="P65" s="2" t="inlineStr">
         <is>
-          <t>Parent's legal counsel; first shown acting 09/20/2021, when it received King &amp; Spalding's revised merger agreement draft.</t>
+          <t>Parent's legal counsel; first shown receiving Kraton's revised draft merger agreement on 09/20/2021.</t>
         </is>
       </c>
       <c r="Q65" s="2" t="inlineStr">
         <is>
-          <t>“O’Melveny &amp; Myers LLP, as counsel to Parent” (p. 39)</t>
+          <t>“King &amp; Spalding LLP provided a revised draft of the merger agreement to O’Melveny &amp; Myers LLP, as counsel to Parent” (p. 39)</t>
         </is>
       </c>
       <c r="R65" s="2" t="n"/>
@@ -4876,12 +4928,14 @@
         <v>1</v>
       </c>
       <c r="G66" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H66" s="4" t="n">
         <v>42</v>
       </c>
-      <c r="I66" s="2" t="n"/>
+      <c r="I66" s="4" t="n">
+        <v>42</v>
+      </c>
       <c r="J66" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
@@ -4904,7 +4958,7 @@
       <c r="O66" s="2" t="n"/>
       <c r="P66" s="2" t="inlineStr">
         <is>
-          <t>Unclear: no condition stated, but Party A's diligence was still open (#59, #67). Formal (markup on file). $42.00 per share plus an earnout paid if the chemical segment is sold above thresholds; Price low only.</t>
+          <t>Unclear: no condition stated, though its next bid “remained” subject to diligence. $42.00 plus an earnout paying extra if the chemical segment sells above thresholds. Formal (markup #55). Revises #59.</t>
         </is>
       </c>
       <c r="Q66" s="2" t="inlineStr">
@@ -4914,7 +4968,7 @@
       </c>
       <c r="R66" s="2" t="inlineStr">
         <is>
-          <t>Q9</t>
+          <t>Q8</t>
         </is>
       </c>
       <c r="S66" s="2" t="n"/>
@@ -4956,7 +5010,7 @@
         <v>1</v>
       </c>
       <c r="G67" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H67" s="2" t="n"/>
       <c r="I67" s="2" t="n"/>
@@ -4970,7 +5024,7 @@
       <c r="O67" s="2" t="n"/>
       <c r="P67" s="2" t="inlineStr">
         <is>
-          <t>Board, citing risks and contingencies and stockholders not sharing fully in chemical-sale value under the earnout, tells Party A its proposal (#65) does not offer adequate value.</t>
+          <t>Board, citing the earnout's risks and contingencies and that stockholders would not share all chemical-sale value, tells J.P. Morgan to inform Party A its proposal is inadequate.</t>
         </is>
       </c>
       <c r="Q67" s="2" t="inlineStr">
@@ -5018,12 +5072,14 @@
         <v>1</v>
       </c>
       <c r="G68" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H68" s="4" t="n">
         <v>44</v>
       </c>
-      <c r="I68" s="2" t="n"/>
+      <c r="I68" s="4" t="n">
+        <v>44</v>
+      </c>
       <c r="J68" s="2" t="inlineStr">
         <is>
           <t>Not stated</t>
@@ -5046,15 +5102,19 @@
       <c r="O68" s="2" t="n"/>
       <c r="P68" s="2" t="inlineStr">
         <is>
-          <t>Light: only confirmatory due diligence. Formal; stated best and final. $44.00 per share plus revised earnout: 50% of net proceeds above thresholds if Kraton agrees to sell the chemical business before closing. Price low only.</t>
+          <t>Light: subject only to confirmatory diligence. $44.00 plus 50% of net chemical-sale proceeds above thresholds if a sale is agreed before closing. Stated as best and final. Formal (markup #55). Revises #65.</t>
         </is>
       </c>
       <c r="Q68" s="2" t="inlineStr">
         <is>
-          <t>“On September 24, 2021, Party A submitted an updated proposal whereby it would acquire Kraton for $44.00 per share.” (p. 40)</t>
-        </is>
-      </c>
-      <c r="R68" s="2" t="n"/>
+          <t>“Party A stated that this proposal was its best and final offer and that it remained subject to confirmatory due diligence.” (p. 40)</t>
+        </is>
+      </c>
+      <c r="R68" s="2" t="inlineStr">
+        <is>
+          <t>Q8</t>
+        </is>
+      </c>
       <c r="S68" s="2" t="n"/>
       <c r="T68" s="3" t="n">
         <v>44463</v>
@@ -5072,42 +5132,48 @@
       </c>
       <c r="B69" s="2" t="inlineStr">
         <is>
-          <t>by 09/27/2021</t>
+          <t>09/27/2021</t>
         </is>
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Goldman Sachs (Asia) L.L.C., Seoul Branch (Parent)</t>
-        </is>
-      </c>
-      <c r="D69" s="2" t="n"/>
+          <t>Parent (DL Chemical Co., Ltd.)</t>
+        </is>
+      </c>
+      <c r="D69" s="2" t="inlineStr">
+        <is>
+          <t>Strategic</t>
+        </is>
+      </c>
       <c r="E69" s="2" t="inlineStr">
         <is>
-          <t>Adviser</t>
+          <t>Other material event</t>
         </is>
       </c>
       <c r="F69" s="2" t="n">
         <v>1</v>
       </c>
       <c r="G69" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H69" s="2" t="n"/>
       <c r="I69" s="2" t="n"/>
       <c r="J69" s="2" t="n"/>
       <c r="K69" s="2" t="n"/>
       <c r="L69" s="2" t="n"/>
-      <c r="M69" s="2" t="n"/>
+      <c r="M69" s="2" t="n">
+        <v>1</v>
+      </c>
       <c r="N69" s="2" t="n"/>
       <c r="O69" s="2" t="n"/>
       <c r="P69" s="2" t="inlineStr">
         <is>
-          <t>Parent's investment banker/broker, from the merger agreement's fees representation (Annex A), not the background. Goldman Sachs Bank USA separately provided Parent's debt commitment (up to $1.75 billion).</t>
+          <t>Financing support: Parent signs a debt commitment letter for up to $1.75 billion with Goldman Sachs Bank USA, the Debt Commitment Party (pp. 7, 42); the merger has no financing condition. From the financing and reasons sections.</t>
         </is>
       </c>
       <c r="Q69" s="2" t="inlineStr">
         <is>
-          <t>“Except for Goldman Sachs (Asia) L.L.C., Seoul Branch, there is no investment banker, broker, finder or other intermediary that has been retained by” (p. A-37)</t>
+          <t>“the financial strength of Parent and Goldman Sachs Bank USA, which provided the Debt Commitment Letter” (p. 42)</t>
         </is>
       </c>
       <c r="R69" s="2" t="n"/>
@@ -5115,7 +5181,9 @@
       <c r="T69" s="3" t="n">
         <v>44466</v>
       </c>
-      <c r="U69" s="2" t="n"/>
+      <c r="U69" s="3" t="n">
+        <v>44466</v>
+      </c>
       <c r="V69" s="3" t="n">
         <v>44466</v>
       </c>
@@ -5131,7 +5199,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Parent (DL Chemical)</t>
+          <t>Parent (DL Chemical Co., Ltd.)</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -5148,7 +5216,7 @@
         <v>1</v>
       </c>
       <c r="G70" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H70" s="2" t="n"/>
       <c r="I70" s="2" t="n"/>
@@ -5162,12 +5230,12 @@
       <c r="O70" s="2" t="n"/>
       <c r="P70" s="2" t="inlineStr">
         <is>
-          <t>$46.50 per share in cash. Board approved 09/26 after J.P. Morgan's fairness opinion. $63 million company termination fee (~4% of equity value); $63 million reverse fee on debt financing failure; no financing condition.</t>
+          <t>$46.50 per share in cash. Signed before market open after Board approval on 09/26 with J.P. Morgan's fairness opinion. $63 million company termination fee (~4% of equity) and $63 million reverse fee on debt financing failure; no-shop with fiduciary out.</t>
         </is>
       </c>
       <c r="Q70" s="2" t="inlineStr">
         <is>
-          <t>“Kraton, Parent, Merger Subsidiary and Intermediate Merger Subsidiary entered into the Merger Agreement” (p. 41)</t>
+          <t>“September 27, 2021, prior to the opening of regular way trading on the NYSE, Kraton, Parent, Merger Subsidiary and Intermediate Merger Subsidiary entered into the Merger Agreement” (p. 41)</t>
         </is>
       </c>
       <c r="R70" s="2" t="n"/>
@@ -5210,7 +5278,7 @@
         <v>1</v>
       </c>
       <c r="G71" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H71" s="2" t="n"/>
       <c r="I71" s="2" t="n"/>
@@ -5228,7 +5296,7 @@
       <c r="O71" s="2" t="n"/>
       <c r="P71" s="2" t="inlineStr">
         <is>
-          <t>Board on 09/26 judged Party A's $44.00-plus-earnout proposal (#67), given its complexity, timing and regulatory risks, not reasonably likely to deliver more value than Parent's.</t>
+          <t>On 09/26 the Board found A's $44.00-plus-earnout offer (#67) not reasonably likely to deliver more value than Parent's $46.50, citing the earnout, complexity, timing and regulatory risk.</t>
         </is>
       </c>
       <c r="Q71" s="2" t="inlineStr">
@@ -5276,7 +5344,7 @@
         <v>1</v>
       </c>
       <c r="G72" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H72" s="2" t="n"/>
       <c r="I72" s="2" t="n"/>
@@ -5298,24 +5366,26 @@
       </c>
       <c r="P72" s="2" t="inlineStr">
         <is>
-          <t>Chemical-segment proposal (#56) still outstanding at signing; the Board had rejected a Sum of the Parts strategy built partly on it. No reported withdrawal.</t>
+          <t>Segment bidder last reported when the Board reviewed its 09/09 proposal on 09/18 and again preferred a whole-company sale; no further mention before signing.</t>
         </is>
       </c>
       <c r="Q72" s="2" t="inlineStr">
         <is>
-          <t>“again determined that a Sum of the Parts Strategy was not likely to deliver greater value for Kraton’s stockholders as compared to what could be achieved” (p. 39)</t>
+          <t>“the Board reviewed the updated proposals submitted by Parent, Party A and Party K” (p. 39)</t>
         </is>
       </c>
       <c r="R72" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="S72" s="2" t="n"/>
       <c r="T72" s="3" t="n">
         <v>44466</v>
       </c>
-      <c r="U72" s="2" t="n"/>
+      <c r="U72" s="3" t="n">
+        <v>44457</v>
+      </c>
       <c r="V72" s="3" t="n">
         <v>44466</v>
       </c>
@@ -5348,7 +5418,7 @@
         <v>1</v>
       </c>
       <c r="G73" s="2" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H73" s="2" t="n"/>
       <c r="I73" s="2" t="n"/>
@@ -5370,7 +5440,7 @@
       </c>
       <c r="P73" s="2" t="inlineStr">
         <is>
-          <t>Party C's $100 million CST proposal (#29) was described as non-withdrawn on 08/30/2021 and never mentioned again; still open at signing.</t>
+          <t>Segment bidder last reported on 08/30 as holding the only other non-withdrawn chemical-segment proposal ($100 million for part of CST); no further mention before signing.</t>
         </is>
       </c>
       <c r="Q73" s="2" t="inlineStr">
@@ -5380,14 +5450,16 @@
       </c>
       <c r="R73" s="2" t="inlineStr">
         <is>
-          <t>Q3</t>
+          <t>Q1</t>
         </is>
       </c>
       <c r="S73" s="2" t="n"/>
       <c r="T73" s="3" t="n">
         <v>44466</v>
       </c>
-      <c r="U73" s="2" t="n"/>
+      <c r="U73" s="3" t="n">
+        <v>44438</v>
+      </c>
       <c r="V73" s="3" t="n">
         <v>44466</v>
       </c>
@@ -5398,132 +5470,60 @@
       </c>
       <c r="B74" s="2" t="inlineStr">
         <is>
-          <t>by 09/27/2021</t>
+          <t>09/27/2021</t>
         </is>
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Post-Reuters financial party</t>
-        </is>
-      </c>
-      <c r="D74" s="2" t="inlineStr">
-        <is>
-          <t>Financial</t>
-        </is>
-      </c>
+          <t>Kraton and Parent</t>
+        </is>
+      </c>
+      <c r="D74" s="2" t="n"/>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Did not submit</t>
+          <t>Merger announced</t>
         </is>
       </c>
       <c r="F74" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G74" s="2" t="n">
-        <v>2</v>
+      <c r="G74" s="2" t="inlineStr">
+        <is>
+          <t>post</t>
+        </is>
       </c>
       <c r="H74" s="2" t="n"/>
       <c r="I74" s="2" t="n"/>
       <c r="J74" s="2" t="n"/>
       <c r="K74" s="2" t="n"/>
       <c r="L74" s="2" t="n"/>
-      <c r="M74" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N74" s="2" t="inlineStr">
-        <is>
-          <t>Not stated</t>
-        </is>
-      </c>
-      <c r="O74" s="2" t="inlineStr">
-        <is>
-          <t>Y</t>
-        </is>
-      </c>
+      <c r="M74" s="2" t="n"/>
+      <c r="N74" s="2" t="n"/>
+      <c r="O74" s="2" t="n"/>
       <c r="P74" s="2" t="inlineStr">
         <is>
-          <t>The filing reports it never submitted a proposal; it was invited to bid (#35) but not included in the 07/20 advancing set. Its exit timing is inferred as by signing, because its NDA date is unknown.</t>
+          <t>Both companies issue press releases announcing the merger agreement on the morning of signing.</t>
         </is>
       </c>
       <c r="Q74" s="2" t="inlineStr">
         <is>
-          <t>“management but did not submit any proposal with respect to a transaction.” (p. 36)</t>
-        </is>
-      </c>
-      <c r="R74" s="2" t="inlineStr">
-        <is>
-          <t>Q6</t>
-        </is>
-      </c>
+          <t>“Kraton and Parent issued press releases announcing execution of the Merger Agreement.” (p. 41)</t>
+        </is>
+      </c>
+      <c r="R74" s="2" t="n"/>
       <c r="S74" s="2" t="n"/>
       <c r="T74" s="3" t="n">
         <v>44466</v>
       </c>
-      <c r="U74" s="2" t="n"/>
+      <c r="U74" s="3" t="n">
+        <v>44466</v>
+      </c>
       <c r="V74" s="3" t="n">
         <v>44466</v>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="2" t="n">
-        <v>74</v>
-      </c>
-      <c r="B75" s="2" t="inlineStr">
-        <is>
-          <t>09/27/2021</t>
-        </is>
-      </c>
-      <c r="C75" s="2" t="inlineStr">
-        <is>
-          <t>Kraton (target)</t>
-        </is>
-      </c>
-      <c r="D75" s="2" t="n"/>
-      <c r="E75" s="2" t="inlineStr">
-        <is>
-          <t>Merger announced</t>
-        </is>
-      </c>
-      <c r="F75" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G75" s="2" t="inlineStr">
-        <is>
-          <t>post</t>
-        </is>
-      </c>
-      <c r="H75" s="2" t="n"/>
-      <c r="I75" s="2" t="n"/>
-      <c r="J75" s="2" t="n"/>
-      <c r="K75" s="2" t="n"/>
-      <c r="L75" s="2" t="n"/>
-      <c r="M75" s="2" t="n"/>
-      <c r="N75" s="2" t="n"/>
-      <c r="O75" s="2" t="n"/>
-      <c r="P75" s="2" t="inlineStr">
-        <is>
-          <t>Kraton and Parent issue press releases before the NYSE open.</t>
-        </is>
-      </c>
-      <c r="Q75" s="2" t="inlineStr">
-        <is>
-          <t>“Kraton and Parent issued press releases announcing execution of the Merger Agreement.” (p. 41)</t>
-        </is>
-      </c>
-      <c r="R75" s="2" t="n"/>
-      <c r="S75" s="2" t="n"/>
-      <c r="T75" s="3" t="n">
-        <v>44466</v>
-      </c>
-      <c r="U75" s="3" t="n">
-        <v>44466</v>
-      </c>
-      <c r="V75" s="3" t="n">
-        <v>44466</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:V75"/>
+  <autoFilter ref="A1:V74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5534,19 +5534,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J5"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
     <col width="7" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
     <col width="40" customWidth="1" min="4" max="4"/>
     <col width="60" customWidth="1" min="5" max="5"/>
     <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
-    <col width="50" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
+    <col width="45" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5613,22 +5613,22 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Board directs outreach to 14 listed buyers and launches the first round (two-phase design)</t>
+          <t>Board directs outreach to 14 listed possible acquirers and commencement of the first round of a two-phase process (#8); outreach end of May–June.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>10 NDA signers: 6 strategic (incl. inbound party; presumed Party A, Parent, Party J, Party K) and 4 financial (presumed Party H, Party I). Segment track: Parties C, D, E, G (strategic, CST only).</t>
+          <t>15 units entered: 11 whole-company confidentiality signers — 6 strategic (Party A, Parent, Party J, Party K [chemical segment only], 2 unnamed; the inbound party is among the six) and 5 financial (Party H, Party I, 2 unnamed, plus 1 unnamed post-Reuters signer after 07/06); and 4 segment-only (CST) strategic parties carried from round 0: Parties C, D, E, G.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>06/29/2021</t>
+          <t>06/29/2021 → 07/19/2021 (updated indications, asked of A, H, Parent and I)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Enforced</t>
+          <t>Extended; Enforced</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
@@ -5638,12 +5638,12 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>4 whole-company: Party A $42–45, Party H $41–43, Parent $41, Party I $40. Other-scope: Party K (chemical segment), Party C and Party G (CST portions).</t>
+          <t>5 whole-company bidders: Party A, Party H, Parent, Party I (by 07/02; A, H, Parent revised by 07/19; I held $40.00) and Party J (by 07/19). Segment proposals: Party K (chemical), Party C and Party G (CST portions).</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>4 whole-company bidders asked to update; 1 NDA signer withdrew; D, E withdrew; J and 3–9 other signers (most likely 3) did not submit</t>
+          <t>3 advanced (Party A, Party H, Parent); Party I and Party J not advanced; 1 strategic signer withdrew; 3 signers and the post-Reuters financial signer never bid; D and E withdrew from CST; C, G, K kept in view.</t>
         </is>
       </c>
     </row>
@@ -5655,26 +5655,26 @@
         <v>2</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>44383</v>
+        <v>44397</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Board requires updated, higher IOIs from the four whole-company bidders before selecting the second round</t>
+          <t>Board invites Party A, Party H and Parent to the second round with additional financial and diligence materials (#46).</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>4 admitted: Party A, Parent (strategic); Party H, Party I (financial). Still being received, not admitted: Party J (bid 07/19); post-Reuters financial NDA signer (invited, no proposal); Parties C, G, K (proposals held, no revision asked).</t>
+          <t>3: 2 strategic (Party A, Parent), 1 financial (Party H). Segment proposals still being received, not admitted: Party C and Party G (CST), Party K (chemical).</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>07/19/2021</t>
+          <t>none stated</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>Enforced</t>
+          <t>No deadline stated</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -5684,12 +5684,12 @@
       </c>
       <c r="I3" s="2" t="inlineStr">
         <is>
-          <t>4: Party A $45, Party H $42–45, Parent $45, Party J $38–41. Party I refused to raise $40.</t>
+          <t>0 (no bids requested; management meetings week of 08/09)</t>
         </is>
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>three advanced (A, H, Parent); I and J out</t>
+          <t>Final bid procedures letter to the same three opens round 3; Party G withdrew 08/04.</t>
         </is>
       </c>
     </row>
@@ -5701,92 +5701,46 @@
         <v>3</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>44397</v>
+        <v>44419</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Board admits Party A, Party H and Parent to the 'second round' with more diligence material</t>
+          <t>Final bid procedures letter after the 08/11 Board authorization of the draft merger agreement (#48).</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>3: Party A, Parent (strategic); Party H (financial). Held segment proposals: Party K, Party C, Party G (G withdrew 08/04).</t>
+          <t>3: 2 strategic (Party A, Parent), 1 financial (Party H). Still being received, not admitted: Party K (chemical; update requested 08/30) and Party C (CST).</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>none stated</t>
+          <t>09/08/2021 (merger agreement markups) → 09/15/2021 (final indications)</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>No deadline stated</t>
+          <t>Passed without action; Late bids accepted</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>Not final</t>
+          <t>Announced as final</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
         <is>
-          <t>0</t>
+          <t>2 whole-company bidders: Parent ($46.00 on 09/15; $46.50 best and final on 09/20) and Party A ($40.50 on 09/17; $42.00 + earnout on 09/21; $44.00 + earnout best and final on 09/24, late after 09/15). Also Party K chemical-segment update (09/09) and Party A polymer-segment alternative (09/17).</t>
         </is>
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>all three sent the final bid procedures letter</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>4</v>
-      </c>
-      <c r="C5" s="3" t="n">
-        <v>44423</v>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>Final bid procedures letter (sent after 08/11, by 08/20): markups due 09/08, final IOIs due 09/15</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>3: Party A, Parent (strategic); Party H (financial). Still being received, not admitted: Party K (updated chemical-segment bid on request, 09/09), Party C (standing CST proposal).</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>09/15/2021 (final IOIs; merger agreement markups separately due 09/08/2021)</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Late bids accepted</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Announced as final</t>
-        </is>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>2: Parent $46.00 then $46.50 (best and final); Party A $40.50 (+ polymer-segment alternative), $42.00 + earnout, $44.00 + earnout (best and final). Other-scope: Party K.</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="inlineStr">
-        <is>
-          <t>signing with Parent 09/27/2021; H withdrew 08/20; A, K, C not selected</t>
+          <t>Signing with Parent 09/27/2021; Party H withdrew 08/20; Party A, Party K and Party C not selected at signing.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J5"/>
+  <autoFilter ref="A1:J4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5797,14 +5751,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="50" customWidth="1" min="2" max="2"/>
-    <col width="50" customWidth="1" min="3" max="3"/>
-    <col width="60" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="45" customWidth="1" min="2" max="2"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
+    <col width="50" customWidth="1" min="4" max="4"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="50" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
@@ -5854,27 +5808,27 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Process and round map: is this one process with four rounds (R1 outreach 05/24; R2 updated-IOI request 07/06; R3 second-round admission 07/20; R4 final bid letter), with the 2020–21 CST divestiture talks as round 0?</t>
+          <t>Should the parties that bid only for parts of Kraton (C, D, E, G for the CST business; K for the chemical segment; A's polymer-segment alternative) be carried as participants, with entries, exits and Other-scope bid rows?</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>Yes. Most plausible alternative: merge R3 and R4 into one 'second round' opened 07/20, with the final letter as a Deadline set (moves round-4 rows #50–#73 to round 3). Less plausible: fold the 07/06 request into round 1 (moves #31–#47).</t>
+          <t>Yes, as segment-only participants. C, D, E and G enter through the 05/20/2021 Board decision to review their CST proposals alongside whole-company bids; K through its round-1 proposal as a confidentiality signer. Their prices stay out of the per-share cells: they are total dollars, enterprise values or EBITDA multiples (mixed bases).</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>E6 counts each selection-and-new-request (07/06, p. 35), each information stage (07/20, p. 36), and the first final-bid request (p. 37) as separate rounds. Gap of about two months or more: CST talks 'late 2020 and early 2021' to end-May 2021 outreach, undated. E5: (a) fails, CST parties still in view (p. 33); (b) not established; (c) met on 05/20. One process.</t>
+          <t>p. 33: Board “would review any proposals submitted by Party C, Party D, Party E, and Party G”; p. 35: on 07/06 C, G, K proposals kept for evaluation; p. 37: 08/30 request for K's update; p. 39: K and A segment proposals reviewed on 09/18.</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>#2, #9, #10, #11, #31, #45, #50</t>
+          <t>#3, #4, #7, #9, #10, #20, #21, #27, #32, #47, #52, #56, #60, #71, #72</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Round counts and finality: merged R3/R4 gives three rounds with the second 'Announced as final'. Merging R2 into R1 treats the 07/19 IOIs as price bargaining rather than a new solicitation.</t>
+          <t>If excluded, round-1 live units fall by four (C, D, E, G) and C, G, K drop out of rounds 2–3; their contact, admission, bid and exit rows would be removed and the Deal facts auction screen is unchanged.</t>
         </is>
       </c>
       <c r="G2" s="2" t="n"/>
@@ -5887,27 +5841,27 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Are the named first-round respondents (Party A, Parent, Party J, Party K; Party H, Party I) members of the 10 NDA signers?</t>
+          <t>Process and round map: one process; round 0 to 05/20/2021; round 1 from 05/24/2021; round 2 from 07/20/2021 (diligence stage); round 3 from the final bid procedures letter after 08/11/2021 to signing. Is this right?</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Treat them as members, as the ledger does: exactly 1 strategic and 2 financial signers did not submit. Counts are left as ranges (1–5, 2–4) because membership is not stated.</t>
+          <t>Keep it. Alternative boundary: merge rounds 2 and 3, reading the 07/20 invitation as the single “second round” named in the filing; #48 would become Deadline set and #47–#72 relabelled round 2. Treating the 07/06 request (#31) as a new round is unsupported (same four bidders, not final). Gaps of about two months or more: possibly between the undated “early 2021” CST talks (#3, #4) and outreach from end of May 2021 (#11–#14), length unknown; none after 05/24/2021. E5 tests for a split before 05/20/2021: (a) fails, C, D, E and G were kept in view (#7); (b) not shown, no reported end and contacts undated; (c) holds, the 05/20 sale decision. One process.</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>The process letter went to each NDA signer and the IOIs came 'as part of the first-round process' (pp. 34–35). The filing never says the named bidders signed NDAs.</t>
+          <t>p. 33: 05/24 Board directed contact of 14 and “to commence the first round”; p. 36: 07/20 invitation to the second round with more diligence; p. 37: “final bid procedures letter” requesting markups and final indications; E6 counts the first request for final offers as a new round.</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>#13, #14, #25, #26, #27, #28</t>
+          <t>#8, #46, #48</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>If some named bidders were not signers, they enter on their bid rows, first-round live units rise by up to six, and more signers did not submit.</t>
+          <t>Merging rounds 2 and 3 gives two Rounds lines instead of three; round 2 would then be Announced as final with due dates 09/08 → 09/15, and G's exit (#47) and all later rows would carry round 2.</t>
         </is>
       </c>
       <c r="G3" s="2" t="n"/>
@@ -5920,27 +5874,27 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Should segment-only parties (Parties C, D, E, G on CST; Party K on the chemical segment) count as live bidder units?</t>
+          <t>Who is inside the 10 confidentiality signers, and are the residual non-submitters (#28, #29) exact?</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Keep them as participants with their own entries and exits, as recorded, but exclude them from whole-company competition in estimation. They can be identified by Other-scope bid rows and the CST/segment Notes.</t>
+          <t>Treat Party A, Parent, Party J and Party K (strategic) and Party H and Party I (financial) as members and keep the exact residuals: 1 strategic and 2 financial signers never bid. The withdrawing signer (#19) is strategic by 6 − 5. Party B's parent may be a signer or a decliner; it is not counted separately in either.</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>The Board said it would weigh CST proposals against whole-company bids (p. 33) and kept C, G and K proposals in view (p. 35). None bid for the whole company.</t>
+          <t>p. 34: 14 listed parties plus one inbound party were contacted; 10 signed (6 strategic, 4 financial) and 5 declined, so all 15 contacts are accounted for; every named party active in round 1 was therefore a signer. p. 34: nine signers (5 strategic, 4 financial) met management.</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>#15, #18, #19, #26, #29, #30, #32, #48, #56, #71, #72</t>
+          <t>#13, #14, #15, #16, #17, #28, #29</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Excluding them drops C, D, E, G and K rows from live counts; whole-company live units at R2 opening fall from 7 to 4.</t>
+          <t>If J or K reached Kraton outside the reported contacts, the strategic residual would be 2–3 and live units in round 1 would rise by up to two; Count on #28 would become a range.</t>
         </is>
       </c>
       <c r="G4" s="2" t="n"/>
@@ -5953,27 +5907,27 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Deadline outcomes: R1 06/29 Enforced; R2 07/19 Enforced; R3 no due date; R4 09/15 Late bids accepted. Are these right?</t>
+          <t>Round 1 deadline outcomes: 06/29/2021 recorded as Extended, 07/19/2021 as Enforced. Correct?</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>Yes. For R1, 'Late bids accepted' is possible if any IOI came 06/30–07/02, but the filing does not show it. The 09/08 markup date is treated as a document deadline, not a bid due date.</t>
+          <t>Keep. On 07/06 the Board gave A, H, Parent and I a later due date (07/19) in the same round after evaluating the bids in hand; on 07/20 it selected three bidders on the bids in hand. Alternative for 06/29: Late bids accepted, since Party J, a signer given the 06/29 date, bid only by 07/19 (#37) and the Board considered it.</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>R1 bids arrived 'By July 2' and the Board acted 07/06 without waiting for Party J (p. 35). R2 responses came 'By July 19' and the Board selected 07/20 (p. 36). Party A bid 09/17, after the 09/15 due date, and the Board reviewed it 09/18 (p. 39).</t>
+          <t>p. 34: process letter asked for initial indications by 06/29; p. 35: indications “By July 2”, J to bid in mid-July, and 07/06 request for updates by 07/19 (printed “2020”); p. 36: 07/20 selection.</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>#20, #38, #57, #59</t>
+          <t>#18, #22, #30, #31, #37, #42</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>If the 09/08 markup date counts as a bid deadline, R4 gets a second outcome (Enforced; both markups on time) and a Deadline row.</t>
+          <t>Deadline outcome for round 1 would read “Late bids accepted; Enforced”; no row or count changes.</t>
         </is>
       </c>
       <c r="G5" s="2" t="n"/>
@@ -5986,27 +5940,27 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Party J missed the 06/29 due date, announced a mid-July bid, and bid $38–$41 on 07/19 without being asked. Is 'Did not submit', then 'Re-entered', right?</t>
+          <t>When did the post-Reuters financial signer enter and leave, and was it live beyond round 1?</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Yes. The alternative keeps J live throughout as a late round-1 bidder, with no exit or re-entry; either way J is out at the 07/20 selection.</t>
+          <t>Record it as a round-1 entrant (confidentiality agreement after 07/06, undated) that never submitted, with the exit sorted at the 07/20 advancement decision, which named a complete set without it; window kept 07/06–09/27.</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>J was not among the four asked for updated IOIs on 07/06 (p. 35); its 07/19 IOI was received (p. 36).</t>
+          <t>pp. 35–36: after the 07/06 Reuters report one financial party “executed a confidentiality agreement … but did not submit any proposal”; p. 36–37: only A, H and Parent received second-round materials and the final bid letter.</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>#25, #43, #44, #47</t>
+          <t>#34, #35, #36, #45</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>Under the alternative, J is live at the R2 opening and its 07/19 bid is round 1, a late bid.</t>
+          <t>If it signed after 07/20 it was never in round 1; it would then be a separate entrant closed as Not selected at signing on 09/27, adding one live unit to rounds 2–3.</t>
         </is>
       </c>
       <c r="G6" s="2" t="n"/>
@@ -6019,27 +5973,27 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Post-Reuters financial NDA signer: what exit label and date?</t>
+          <t>How should Party I's and Party J's departures at the 07/20 selection be labelled?</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>'Did not submit' by signing (09/27), round 2, as recorded. If its NDA preceded 07/20, 'Dropped by target' on 07/20 is equally defensible.</t>
+          <t>Both Dropped by target (inferred: the complete advancing set A, H, Parent is named). Party I: Would not improve earlier offer, because it was asked on 07/06 for a higher value and refused. Party J: Not stated; it said it would not go above $41.00 but was never asked to improve.</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>It signed an NDA and met management after 07/06 but 'did not submit any proposal' (pp. 35–36). Its dates are not given.</t>
+          <t>p. 35: Board required updated indications from A, H, Parent and I; p. 36: I “not willing to increase” $40.00, J “not willing to increase its purchase price beyond this range”; 07/20 invitation to A, H and Parent only.</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>#36, #37, #73</t>
+          <t>#41, #43, #44</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>A 07/20 drop would remove it from live units in rounds 3–4 (live units at R4 opening 6 → 5).</t>
+          <t>J could instead take Would not improve earlier offer or Lower offer than rivals, which records its valuation cap of $41.00 for the model; I's reason could fall to Not stated.</t>
         </is>
       </c>
       <c r="G7" s="2" t="n"/>
@@ -6052,27 +6006,27 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Party I's inferred 07/20 drop: should the exit reason be 'Would not improve earlier offer' or 'Not stated'?</t>
+          <t>Round 3 deadline outcomes: 09/08/2021 (markups) Passed without action; 09/15/2021 (final indications) Late bids accepted. Correct?</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>'Would not improve earlier offer'. Party I was asked for greater value and refused to raise $40.00.</t>
+          <t>Keep. Both remaining bidders delivered markups on 09/08 and bidding continued to 09/15; Parent bid on 09/15, Party A only on 09/17, and the Board reviewed A's late bid on 09/18.</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>E14 gives this reason to a bidder asked to improve that declines, even where the target then chooses rivals. The refusal is reported (p. 36).</t>
+          <t>p. 37: letter requested markups by 09/08 and final indications by 09/15; p. 38: markups 09/08; p. 39: Parent 09/15, A 09/17, Board review 09/18.</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>#42, #46</t>
+          <t>#48, #53, #58, #59</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>'Not stated' would lose the valuation signal (I's value is about $40).</t>
+          <t>If the markup date is not treated as a bid due date, 09/08 loses its Deadline row and outcome; reading 09/18 as action on the bids in hand would make 09/15 Enforced.</t>
         </is>
       </c>
       <c r="G8" s="2" t="n"/>
@@ -6085,66 +6039,33 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Should the 09/08 merger agreement markups be Bid rows carrying the 07/19 price, rather than Other material events?</t>
+          <t>Formality and conditions of the round-3 offers: markups as Other material event rows; Parent 09/15 and 09/20 Formal/Light; A 09/17 Formal/Heavy, 09/21 Formal/Unclear, 09/24 Formal/Light; A's polymer alternative Informal/Heavy.</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>No. Record them as events and make the next priced offers (09/15 Parent, 09/17 Party A) the first Formal bids.</t>
+          <t>Keep. The 09/08 markups carried no new price, so they support later bids rather than forming Bid rows. Parent had substantially completed diligence and financing was not a condition; A's 09/24 bid named only confirmatory diligence.</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Neither markup came with a price (p. 38). E11 needs a markup with a priced proposal or in support of one; the prices followed a week later.</t>
+          <t>p. 38: Parent's markup (no financing condition, but it required debt financing); Parent “completed substantially all due diligence”; p. 39: A's 09/17 bid “subject to additional due diligence”; p. 40: A 09/24 “subject to confirmatory due diligence”; Board cited regulatory risks.</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>#54, #55, #58</t>
+          <t>#54, #55, #57, #59, #60, #63, #65, #67</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>As Bid rows, Parent's and Party A's $45.00 would become Formal from 09/08, a week earlier.</t>
+          <t>Parent's bids become Heavy if the unsigned debt commitment (letter still in draft on 09/20) counts as reported absence of commitment; A's 09/24 becomes Heavy if the Board's regulatory-risk concern is an identified obstacle; A's 09/17 becomes Light if “additional” means confirmatory.</t>
         </is>
       </c>
       <c r="G9" s="2" t="n"/>
     </row>
-    <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Q9</t>
-        </is>
-      </c>
-      <c r="B10" s="2" t="inlineStr">
-        <is>
-          <t>Conditions on Party A's 09/17 and 09/21 bids: Heavy and Unclear?</t>
-        </is>
-      </c>
-      <c r="C10" s="2" t="inlineStr">
-        <is>
-          <t>Yes. 09/17 'subject to additional due diligence' is Heavy (open-ended, unlike the later 'confirmatory'). 09/21 states no condition while diligence remained open: Unclear.</t>
-        </is>
-      </c>
-      <c r="D10" s="2" t="inlineStr">
-        <is>
-          <t>On 09/24 Party A described its diligence as confirmatory (p. 40). The 09/17 wording is broader (p. 39). The Board cited 'risks and contingencies' on 09/23 (p. 40).</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>#59, #65</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Light on 09/17 would make Party A's first final-round bid a low-conditionality bid at $40.50.</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="n"/>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G10"/>
+  <autoFilter ref="A1:G9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6182,7 +6103,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Kraton Corporation (NYSE: KRA), Houston, Texas; specialty polymers and pine-based chemicals</t>
+          <t>Kraton Corporation (NYSE: KRA), Houston, Texas; polymer and chemical segments</t>
         </is>
       </c>
     </row>
@@ -6194,7 +6115,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>DL Chemical Co., Ltd. (Parent), a DL Holdings Co., Ltd. subsidiary, through DLC US Holdings, Inc. and DLC US, Inc.</t>
+          <t>DL Chemical Co., Ltd. (“Parent”), Seoul, South Korea, a subsidiary of DL Holdings Co., Ltd., through DLC US Holdings, Inc. and DLC US, Inc.</t>
         </is>
       </c>
     </row>
@@ -6206,7 +6127,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Strategic (South Korean petrochemical operating company)</t>
+          <t>Strategic</t>
         </is>
       </c>
     </row>
@@ -6218,7 +6139,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>$46.50 per share in cash; funded with up to $1.75 billion committed debt from Goldman Sachs Bank USA and Parent cash; no financing condition; $63 million termination and reverse termination fees</t>
+          <t>$46.50 per share in cash, without interest; about $2.5 billion of total funds (including refinancing of Kraton debt), from up to $1.75 billion of committed debt financing (Goldman Sachs Bank USA) and Parent's cash; no financing condition</t>
         </is>
       </c>
     </row>
@@ -6242,7 +6163,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>09/27/2021 (press releases before the NYSE open)</t>
+          <t>09/27/2021</t>
         </is>
       </c>
     </row>
@@ -6254,7 +6175,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>DEFM14A definitive proxy statement, dated 11/04/2021</t>
+          <t>DEFM14A (definitive proxy statement), 11/04/2021</t>
         </is>
       </c>
     </row>
@@ -6302,7 +6223,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>None reported. Before the 05/20/2021 sale decision, Kraton's 12/2020 corporate development plan sought polymer acquisitions (Parties A and B declined; no rows) and a CST divestiture (Parties C–G; recorded as round 0).</t>
+          <t>None reported for the whole company. From December 2020 Kraton pursued a corporate development plan: buying or combining with the polymer businesses of Parties A and B (both declined) and selling its CST business (Parties C, D, E, F, G approached); the CST track carried into process 1 as round 0 (#2–#4, #7). Parent had bought Kraton's Cariflex business in March 2020.</t>
         </is>
       </c>
     </row>
@@ -6314,7 +6235,7 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Met (process 1): 11 parties (10 by late June 2021, 6 strategic and 4 financial, plus 1 post-Reuters financial party)</t>
+          <t>Met (process 1): 11 parties (10 by late June 2021 — 6 strategic, 4 financial — plus 1 financial party after 07/06/2021)</t>
         </is>
       </c>
     </row>
@@ -6326,7 +6247,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Yes. Also other-scope bids: Party K (chemical segment), Parties C and G (portions of the CST business), Party A's alternative (polymer segment with chemical spin-off)</t>
+          <t>Yes (also segment bids: Parties C and G for portions of the CST business, Party K for the chemical segment, Party A's alternative for the polymer segment)</t>
         </is>
       </c>
     </row>
@@ -6338,7 +6259,7 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>US dollars per share for whole-company bids. Segment bids are stated as totals, EBITDA multiples or enterprise values (see Notes). Party A bids of 09/21 and 09/24 add an unquantified earnout.</t>
+          <t>US dollars per share for whole-company bids; segment bids in total US dollars, enterprise value or multiples of segment EBITDA (mixed bases; see Q1). Party A's last two bids add an earnout to the per-share price.</t>
         </is>
       </c>
     </row>
@@ -6374,7 +6295,7 @@
       </c>
       <c r="B18" s="2" t="inlineStr">
         <is>
-          <t>After a 2020 strategy review, Kraton sought polymer acquisitions and a sale of its CST business; the effort stalled, and on 05/20/2021 the Board decided to explore a sale of the whole company. J.P. Morgan contacted 14 listed buyers plus one inbound party, and 10 signed NDAs. Four whole-company IOIs ($40–$45) arrived by early July, alongside segment bids from Parties K, C and G. After a round of updated IOIs, Party A, Party H and Parent were taken to a final round; Party H withdrew on 08/20, unable to hold its range. Parent bid $46.00 on 09/15 and, when asked, raised to $46.50 best and final; Party A's lower bids ($40.50, then $42.00 and $44.00 with earnouts) were rejected. Kraton and Parent signed on 09/27/2021 at $46.50 in cash.</t>
+          <t>After a corporate development plan to buy polymer businesses and sell the CST business stalled, Kraton's board decided on 05/20/2021 to explore a sale of the whole company. J.P. Morgan contacted 14 listed parties and received one inbound inquiry; 10 signed confidentiality agreements, and one more financial party signed after a 07/06 Reuters leak. Four indications arrived by early July (Party A $42–45, H $41–43, Parent $41, I $40), and after a request for higher values the board advanced A, H and Parent on 07/20, dropping I and late bidder J. H withdrew on 08/20; in the final round Parent bid $46.00 and then, at the board's request, $46.50 best and final, while Party A bid $40.50 and then $42.00 and $44.00 with chemical-segment earnouts. Segment offers from Parties C, G and K were weighed as a sum-of-the-parts alternative and rejected, and Kraton signed with Parent on 09/27/2021 at $46.50 in cash.</t>
         </is>
       </c>
     </row>

</xml_diff>